<commit_message>
Review sheet: mark modified Process entries in green font
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_review/Potential_Revisione_Traduzioni.xlsx
+++ b/_review/Potential_Revisione_Traduzioni.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -50,6 +50,11 @@
       <family val="2"/>
       <color rgb="FF999999"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001E7D32"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="5">
@@ -102,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -128,6 +133,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3579,27 +3590,27 @@
           <t>pr-t1</t>
         </is>
       </c>
-      <c r="B104" s="9" t="inlineStr">
+      <c r="B104" s="11" t="inlineStr">
         <is>
           <t>Pre-Construction &amp; Audit</t>
         </is>
       </c>
-      <c r="C104" s="9" t="inlineStr">
+      <c r="C104" s="11" t="inlineStr">
         <is>
           <t>Pre-Construction &amp; Audit</t>
         </is>
       </c>
-      <c r="D104" s="9" t="inlineStr">
+      <c r="D104" s="11" t="inlineStr">
         <is>
           <t>施工前审核</t>
         </is>
       </c>
-      <c r="E104" s="9" t="inlineStr">
+      <c r="E104" s="11" t="inlineStr">
         <is>
           <t>Подготовка и аудит</t>
         </is>
       </c>
-      <c r="F104" s="10" t="inlineStr">
+      <c r="F104" s="12" t="inlineStr">
         <is>
           <t>التحضير والتدقيق</t>
         </is>
@@ -3611,27 +3622,27 @@
           <t>pr-i1a</t>
         </is>
       </c>
-      <c r="B105" s="9" t="inlineStr">
+      <c r="B105" s="11" t="inlineStr">
         <is>
           <t>Drawing &amp; spec review</t>
         </is>
       </c>
-      <c r="C105" s="9" t="inlineStr">
+      <c r="C105" s="11" t="inlineStr">
         <is>
           <t>Revisione disegni e capitolati</t>
         </is>
       </c>
-      <c r="D105" s="9" t="inlineStr">
+      <c r="D105" s="11" t="inlineStr">
         <is>
           <t>图纸与规范审查</t>
         </is>
       </c>
-      <c r="E105" s="9" t="inlineStr">
+      <c r="E105" s="11" t="inlineStr">
         <is>
           <t>Проверка чертежей и спецификаций</t>
         </is>
       </c>
-      <c r="F105" s="10" t="inlineStr">
+      <c r="F105" s="12" t="inlineStr">
         <is>
           <t>مراجعة الرسومات والمواصفات</t>
         </is>
@@ -3675,27 +3686,27 @@
           <t>pr-i1c</t>
         </is>
       </c>
-      <c r="B107" s="9" t="inlineStr">
+      <c r="B107" s="11" t="inlineStr">
         <is>
           <t>RFI risk log</t>
         </is>
       </c>
-      <c r="C107" s="9" t="inlineStr">
+      <c r="C107" s="11" t="inlineStr">
         <is>
           <t>Registro RFI e rischi</t>
         </is>
       </c>
-      <c r="D107" s="9" t="inlineStr">
+      <c r="D107" s="11" t="inlineStr">
         <is>
           <t>RFI 风险记录</t>
         </is>
       </c>
-      <c r="E107" s="9" t="inlineStr">
+      <c r="E107" s="11" t="inlineStr">
         <is>
           <t>Журнал RFI и рисков</t>
         </is>
       </c>
-      <c r="F107" s="10" t="inlineStr">
+      <c r="F107" s="12" t="inlineStr">
         <is>
           <t>سجل RFI والمخاطر</t>
         </is>
@@ -3707,27 +3718,27 @@
           <t>pr-i1d</t>
         </is>
       </c>
-      <c r="B108" s="9" t="inlineStr">
+      <c r="B108" s="11" t="inlineStr">
         <is>
           <t>Value engineering</t>
         </is>
       </c>
-      <c r="C108" s="9" t="inlineStr">
+      <c r="C108" s="11" t="inlineStr">
         <is>
           <t>Value engineering</t>
         </is>
       </c>
-      <c r="D108" s="9" t="inlineStr">
+      <c r="D108" s="11" t="inlineStr">
         <is>
           <t>价值工程</t>
         </is>
       </c>
-      <c r="E108" s="9" t="inlineStr">
+      <c r="E108" s="11" t="inlineStr">
         <is>
           <t>Стоимостной инжиниринг</t>
         </is>
       </c>
-      <c r="F108" s="10" t="inlineStr">
+      <c r="F108" s="12" t="inlineStr">
         <is>
           <t>هندسة القيمة</t>
         </is>
@@ -3739,27 +3750,27 @@
           <t>pr-t2</t>
         </is>
       </c>
-      <c r="B109" s="9" t="inlineStr">
+      <c r="B109" s="11" t="inlineStr">
         <is>
           <t>Bid &amp; Buyout</t>
         </is>
       </c>
-      <c r="C109" s="9" t="inlineStr">
+      <c r="C109" s="11" t="inlineStr">
         <is>
           <t>Bid &amp; Buyout</t>
         </is>
       </c>
-      <c r="D109" s="9" t="inlineStr">
+      <c r="D109" s="11" t="inlineStr">
         <is>
           <t>招标与采购</t>
         </is>
       </c>
-      <c r="E109" s="9" t="inlineStr">
+      <c r="E109" s="11" t="inlineStr">
         <is>
           <t>Тендер и закупки</t>
         </is>
       </c>
-      <c r="F109" s="10" t="inlineStr">
+      <c r="F109" s="12" t="inlineStr">
         <is>
           <t>المناقصة والشراء</t>
         </is>
@@ -3771,27 +3782,27 @@
           <t>pr-i2a</t>
         </is>
       </c>
-      <c r="B110" s="9" t="inlineStr">
+      <c r="B110" s="11" t="inlineStr">
         <is>
           <t>Bid solicitation</t>
         </is>
       </c>
-      <c r="C110" s="9" t="inlineStr">
+      <c r="C110" s="11" t="inlineStr">
         <is>
           <t>Bando di gara</t>
         </is>
       </c>
-      <c r="D110" s="9" t="inlineStr">
+      <c r="D110" s="11" t="inlineStr">
         <is>
           <t>招标公告</t>
         </is>
       </c>
-      <c r="E110" s="9" t="inlineStr">
+      <c r="E110" s="11" t="inlineStr">
         <is>
           <t>Объявление тендера</t>
         </is>
       </c>
-      <c r="F110" s="10" t="inlineStr">
+      <c r="F110" s="12" t="inlineStr">
         <is>
           <t>طرح المناقصة</t>
         </is>
@@ -3803,27 +3814,27 @@
           <t>pr-i2b</t>
         </is>
       </c>
-      <c r="B111" s="9" t="inlineStr">
+      <c r="B111" s="11" t="inlineStr">
         <is>
           <t>Subcontractor prequalification</t>
         </is>
       </c>
-      <c r="C111" s="9" t="inlineStr">
+      <c r="C111" s="11" t="inlineStr">
         <is>
           <t>Prequalifica subappaltatori</t>
         </is>
       </c>
-      <c r="D111" s="9" t="inlineStr">
+      <c r="D111" s="11" t="inlineStr">
         <is>
           <t>分包商预审</t>
         </is>
       </c>
-      <c r="E111" s="9" t="inlineStr">
+      <c r="E111" s="11" t="inlineStr">
         <is>
           <t>Предквалификация субподрядчиков</t>
         </is>
       </c>
-      <c r="F111" s="10" t="inlineStr">
+      <c r="F111" s="12" t="inlineStr">
         <is>
           <t>التأهيل المسبق للمقاولين من الباطن</t>
         </is>
@@ -3835,27 +3846,27 @@
           <t>pr-i2c</t>
         </is>
       </c>
-      <c r="B112" s="9" t="inlineStr">
+      <c r="B112" s="11" t="inlineStr">
         <is>
           <t>Bid leveling</t>
         </is>
       </c>
-      <c r="C112" s="9" t="inlineStr">
+      <c r="C112" s="11" t="inlineStr">
         <is>
           <t>Bid leveling</t>
         </is>
       </c>
-      <c r="D112" s="9" t="inlineStr">
+      <c r="D112" s="11" t="inlineStr">
         <is>
           <t>报价比选</t>
         </is>
       </c>
-      <c r="E112" s="9" t="inlineStr">
+      <c r="E112" s="11" t="inlineStr">
         <is>
           <t>Bid leveling</t>
         </is>
       </c>
-      <c r="F112" s="10" t="inlineStr">
+      <c r="F112" s="12" t="inlineStr">
         <is>
           <t>Bid leveling</t>
         </is>
@@ -3867,27 +3878,27 @@
           <t>pr-i2d</t>
         </is>
       </c>
-      <c r="B113" s="9" t="inlineStr">
+      <c r="B113" s="11" t="inlineStr">
         <is>
           <t>Award recommendation</t>
         </is>
       </c>
-      <c r="C113" s="9" t="inlineStr">
+      <c r="C113" s="11" t="inlineStr">
         <is>
           <t>Proposta di aggiudicazione</t>
         </is>
       </c>
-      <c r="D113" s="9" t="inlineStr">
+      <c r="D113" s="11" t="inlineStr">
         <is>
           <t>授标建议</t>
         </is>
       </c>
-      <c r="E113" s="9" t="inlineStr">
+      <c r="E113" s="11" t="inlineStr">
         <is>
           <t>Рекомендация по присуждению</t>
         </is>
       </c>
-      <c r="F113" s="10" t="inlineStr">
+      <c r="F113" s="12" t="inlineStr">
         <is>
           <t>توصية الإرساء</t>
         </is>
@@ -3899,27 +3910,27 @@
           <t>pr-t3</t>
         </is>
       </c>
-      <c r="B114" s="9" t="inlineStr">
+      <c r="B114" s="11" t="inlineStr">
         <is>
           <t>Contract Award</t>
         </is>
       </c>
-      <c r="C114" s="9" t="inlineStr">
+      <c r="C114" s="11" t="inlineStr">
         <is>
           <t>Aggiudicazione</t>
         </is>
       </c>
-      <c r="D114" s="9" t="inlineStr">
+      <c r="D114" s="11" t="inlineStr">
         <is>
           <t>合同授予</t>
         </is>
       </c>
-      <c r="E114" s="9" t="inlineStr">
+      <c r="E114" s="11" t="inlineStr">
         <is>
           <t>Заключение договора</t>
         </is>
       </c>
-      <c r="F114" s="10" t="inlineStr">
+      <c r="F114" s="12" t="inlineStr">
         <is>
           <t>إرساء العقد</t>
         </is>
@@ -3931,27 +3942,27 @@
           <t>pr-i3a</t>
         </is>
       </c>
-      <c r="B115" s="9" t="inlineStr">
+      <c r="B115" s="11" t="inlineStr">
         <is>
           <t>Scope of Work review</t>
         </is>
       </c>
-      <c r="C115" s="9" t="inlineStr">
+      <c r="C115" s="11" t="inlineStr">
         <is>
           <t>Revisione Scope of Work</t>
         </is>
       </c>
-      <c r="D115" s="9" t="inlineStr">
+      <c r="D115" s="11" t="inlineStr">
         <is>
           <t>工作范围审查</t>
         </is>
       </c>
-      <c r="E115" s="9" t="inlineStr">
+      <c r="E115" s="11" t="inlineStr">
         <is>
           <t>Проверка объёма работ</t>
         </is>
       </c>
-      <c r="F115" s="10" t="inlineStr">
+      <c r="F115" s="12" t="inlineStr">
         <is>
           <t>مراجعة نطاق العمل</t>
         </is>
@@ -3963,27 +3974,27 @@
           <t>pr-i3b</t>
         </is>
       </c>
-      <c r="B116" s="9" t="inlineStr">
+      <c r="B116" s="11" t="inlineStr">
         <is>
           <t>Schedule of Values</t>
         </is>
       </c>
-      <c r="C116" s="9" t="inlineStr">
+      <c r="C116" s="11" t="inlineStr">
         <is>
           <t>Schedule of Values</t>
         </is>
       </c>
-      <c r="D116" s="9" t="inlineStr">
+      <c r="D116" s="11" t="inlineStr">
         <is>
           <t>Schedule of Values</t>
         </is>
       </c>
-      <c r="E116" s="9" t="inlineStr">
+      <c r="E116" s="11" t="inlineStr">
         <is>
           <t>Schedule of Values</t>
         </is>
       </c>
-      <c r="F116" s="10" t="inlineStr">
+      <c r="F116" s="12" t="inlineStr">
         <is>
           <t>Schedule of Values</t>
         </is>
@@ -3995,27 +4006,27 @@
           <t>pr-i3c</t>
         </is>
       </c>
-      <c r="B117" s="9" t="inlineStr">
+      <c r="B117" s="11" t="inlineStr">
         <is>
           <t>Liquidated damages</t>
         </is>
       </c>
-      <c r="C117" s="9" t="inlineStr">
+      <c r="C117" s="11" t="inlineStr">
         <is>
           <t>Penali contrattuali</t>
         </is>
       </c>
-      <c r="D117" s="9" t="inlineStr">
+      <c r="D117" s="11" t="inlineStr">
         <is>
           <t>违约金</t>
         </is>
       </c>
-      <c r="E117" s="9" t="inlineStr">
+      <c r="E117" s="11" t="inlineStr">
         <is>
           <t>Неустойка</t>
         </is>
       </c>
-      <c r="F117" s="10" t="inlineStr">
+      <c r="F117" s="12" t="inlineStr">
         <is>
           <t>غرامات التأخير</t>
         </is>
@@ -4123,27 +4134,27 @@
           <t>pr-i4b</t>
         </is>
       </c>
-      <c r="B121" s="9" t="inlineStr">
+      <c r="B121" s="11" t="inlineStr">
         <is>
           <t>Progress meetings</t>
         </is>
       </c>
-      <c r="C121" s="9" t="inlineStr">
+      <c r="C121" s="11" t="inlineStr">
         <is>
           <t>Riunioni di avanzamento</t>
         </is>
       </c>
-      <c r="D121" s="9" t="inlineStr">
+      <c r="D121" s="11" t="inlineStr">
         <is>
           <t>进度会议</t>
         </is>
       </c>
-      <c r="E121" s="9" t="inlineStr">
+      <c r="E121" s="11" t="inlineStr">
         <is>
           <t>Совещания по ходу работ</t>
         </is>
       </c>
-      <c r="F121" s="10" t="inlineStr">
+      <c r="F121" s="12" t="inlineStr">
         <is>
           <t>اجتماعات المتابعة</t>
         </is>
@@ -4155,27 +4166,27 @@
           <t>pr-i4c</t>
         </is>
       </c>
-      <c r="B122" s="9" t="inlineStr">
+      <c r="B122" s="11" t="inlineStr">
         <is>
           <t>Change order log</t>
         </is>
       </c>
-      <c r="C122" s="9" t="inlineStr">
+      <c r="C122" s="11" t="inlineStr">
         <is>
           <t>Registro varianti</t>
         </is>
       </c>
-      <c r="D122" s="9" t="inlineStr">
+      <c r="D122" s="11" t="inlineStr">
         <is>
           <t>变更单记录</t>
         </is>
       </c>
-      <c r="E122" s="9" t="inlineStr">
+      <c r="E122" s="11" t="inlineStr">
         <is>
           <t>Журнал изменений</t>
         </is>
       </c>
-      <c r="F122" s="10" t="inlineStr">
+      <c r="F122" s="12" t="inlineStr">
         <is>
           <t>سجل أوامر التغيير</t>
         </is>
@@ -4219,27 +4230,27 @@
           <t>pr-t5</t>
         </is>
       </c>
-      <c r="B124" s="9" t="inlineStr">
+      <c r="B124" s="11" t="inlineStr">
         <is>
           <t>Closeout &amp; Turnover</t>
         </is>
       </c>
-      <c r="C124" s="9" t="inlineStr">
+      <c r="C124" s="11" t="inlineStr">
         <is>
           <t>Closeout &amp; Turnover</t>
         </is>
       </c>
-      <c r="D124" s="9" t="inlineStr">
+      <c r="D124" s="11" t="inlineStr">
         <is>
           <t>竣工与移交</t>
         </is>
       </c>
-      <c r="E124" s="9" t="inlineStr">
+      <c r="E124" s="11" t="inlineStr">
         <is>
           <t>Закрытие и передача</t>
         </is>
       </c>
-      <c r="F124" s="10" t="inlineStr">
+      <c r="F124" s="12" t="inlineStr">
         <is>
           <t>الإغلاق والتسليم</t>
         </is>
@@ -4251,27 +4262,27 @@
           <t>pr-i5a</t>
         </is>
       </c>
-      <c r="B125" s="9" t="inlineStr">
+      <c r="B125" s="11" t="inlineStr">
         <is>
           <t>Substantial completion</t>
         </is>
       </c>
-      <c r="C125" s="9" t="inlineStr">
+      <c r="C125" s="11" t="inlineStr">
         <is>
           <t>Substantial completion</t>
         </is>
       </c>
-      <c r="D125" s="9" t="inlineStr">
+      <c r="D125" s="11" t="inlineStr">
         <is>
           <t>实质性竣工</t>
         </is>
       </c>
-      <c r="E125" s="9" t="inlineStr">
+      <c r="E125" s="11" t="inlineStr">
         <is>
           <t>Существенное завершение</t>
         </is>
       </c>
-      <c r="F125" s="10" t="inlineStr">
+      <c r="F125" s="12" t="inlineStr">
         <is>
           <t>الإنجاز الجوهري</t>
         </is>
@@ -4315,27 +4326,27 @@
           <t>pr-i5c</t>
         </is>
       </c>
-      <c r="B127" s="9" t="inlineStr">
+      <c r="B127" s="11" t="inlineStr">
         <is>
           <t>As-built documentation</t>
         </is>
       </c>
-      <c r="C127" s="9" t="inlineStr">
+      <c r="C127" s="11" t="inlineStr">
         <is>
           <t>Documentazione as-built</t>
         </is>
       </c>
-      <c r="D127" s="9" t="inlineStr">
+      <c r="D127" s="11" t="inlineStr">
         <is>
           <t>竣工图文件</t>
         </is>
       </c>
-      <c r="E127" s="9" t="inlineStr">
+      <c r="E127" s="11" t="inlineStr">
         <is>
           <t>Исполнительная документация</t>
         </is>
       </c>
-      <c r="F127" s="10" t="inlineStr">
+      <c r="F127" s="12" t="inlineStr">
         <is>
           <t>مخططات كما نُفِّذت</t>
         </is>
@@ -4347,27 +4358,27 @@
           <t>pr-i5d</t>
         </is>
       </c>
-      <c r="B128" s="9" t="inlineStr">
+      <c r="B128" s="11" t="inlineStr">
         <is>
           <t>Warranty &amp; O&amp;M manuals</t>
         </is>
       </c>
-      <c r="C128" s="9" t="inlineStr">
+      <c r="C128" s="11" t="inlineStr">
         <is>
           <t>Garanzie e manuali O&amp;M</t>
         </is>
       </c>
-      <c r="D128" s="9" t="inlineStr">
+      <c r="D128" s="11" t="inlineStr">
         <is>
           <t>保修与运维手册</t>
         </is>
       </c>
-      <c r="E128" s="9" t="inlineStr">
+      <c r="E128" s="11" t="inlineStr">
         <is>
           <t>Гарантии и руководства по эксплуатации</t>
         </is>
       </c>
-      <c r="F128" s="10" t="inlineStr">
+      <c r="F128" s="12" t="inlineStr">
         <is>
           <t>الضمانات وأدلة التشغيل والصيانة</t>
         </is>
@@ -4719,8 +4730,8 @@
     <mergeCell ref="A129:F129"/>
     <mergeCell ref="A11:F11"/>
     <mergeCell ref="A138:F138"/>
+    <mergeCell ref="A1:F1"/>
     <mergeCell ref="A80:F80"/>
-    <mergeCell ref="A1:F1"/>
     <mergeCell ref="A94:F94"/>
     <mergeCell ref="A103:F103"/>
     <mergeCell ref="A134:F134"/>

</xml_diff>

<commit_message>
Review sheet: add 'Numeri' tab to edit statistics figures
</commit_message>
<xml_diff>
--- a/_review/Potential_Revisione_Traduzioni.xlsx
+++ b/_review/Potential_Revisione_Traduzioni.xlsx
@@ -7,6 +7,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traduzioni" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Numeri" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -16,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,9 +53,35 @@
       <sz val="9"/>
     </font>
     <font>
+      <name val="Calibri (Corpo)"/>
+      <color theme="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
       <name val="Calibri"/>
+      <family val="2"/>
+      <color rgb="FFC00000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="00999999"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="001E7D32"/>
-      <sz val="11"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="5">
@@ -76,11 +103,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF3C4"/>
+        <fgColor rgb="00C71617"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -103,11 +130,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00DDDDDD"/>
+      </left>
+      <right style="thin">
+        <color rgb="00DDDDDD"/>
+      </right>
+      <top style="thin">
+        <color rgb="00DDDDDD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00DDDDDD"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -122,6 +163,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -129,17 +179,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -509,12 +558,12 @@
   <dimension ref="A1:F141"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" style="7" min="1" max="1"/>
-    <col width="34" customWidth="1" style="7" min="2" max="6"/>
+    <col width="16" customWidth="1" style="10" min="1" max="1"/>
+    <col width="34" customWidth="1" style="10" min="2" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" s="7">
-      <c r="A1" s="8" t="inlineStr">
+    <row r="1" ht="34" customHeight="1" s="10">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Potential — Revisione traduzioni  ·  Modifica le celle di lingua (non la colonna ID). Le righe rosse sono i titoli di sezione (ordine del sito). Simboli &lt;br&gt;/&lt;em&gt; = a capo/evidenziazioni, lasciarli.</t>
         </is>
@@ -552,14 +601,14 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="20" customHeight="1" s="7">
-      <c r="A3" s="6" t="inlineStr">
+    <row r="3" ht="20" customHeight="1" s="10">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Elementi ricorrenti (scroll, footer)</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="16" customHeight="1" s="7">
+    <row r="4" ht="16" customHeight="1" s="10">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>scroll-down</t>
@@ -591,7 +640,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="16" customHeight="1" s="7">
+    <row r="5" ht="16" customHeight="1" s="10">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>footer-copy</t>
@@ -623,7 +672,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="16" customHeight="1" s="7">
+    <row r="6" ht="16" customHeight="1" s="10">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>footer-privacy</t>
@@ -655,14 +704,14 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="20" customHeight="1" s="7">
-      <c r="A7" s="6" t="inlineStr">
+    <row r="7" ht="20" customHeight="1" s="10">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>1 · Frase d'apertura</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="16" customHeight="1" s="7">
+    <row r="8" ht="16" customHeight="1" s="10">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>intro-hl-1</t>
@@ -694,7 +743,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="16" customHeight="1" s="7">
+    <row r="9" ht="16" customHeight="1" s="10">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>intro-hl-2</t>
@@ -726,7 +775,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="16" customHeight="1" s="7">
+    <row r="10" ht="16" customHeight="1" s="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>intro-hl-3</t>
@@ -758,14 +807,14 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="20" customHeight="1" s="7">
-      <c r="A11" s="6" t="inlineStr">
+    <row r="11" ht="20" customHeight="1" s="10">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>2 · Aree di competenza</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="16" customHeight="1" s="7">
+    <row r="12" ht="16" customHeight="1" s="10">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>stag-coverage</t>
@@ -797,7 +846,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="32" customHeight="1" s="7">
+    <row r="13" ht="32" customHeight="1" s="10">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>sectors-hl</t>
@@ -829,7 +878,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="16" customHeight="1" s="7">
+    <row r="14" ht="16" customHeight="1" s="10">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>s01-title</t>
@@ -861,7 +910,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="16" customHeight="1" s="7">
+    <row r="15" ht="16" customHeight="1" s="10">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>s01-i1</t>
@@ -893,7 +942,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="16" customHeight="1" s="7">
+    <row r="16" ht="16" customHeight="1" s="10">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>s01-i2</t>
@@ -925,7 +974,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="16" customHeight="1" s="7">
+    <row r="17" ht="16" customHeight="1" s="10">
       <c r="A17" s="3" t="inlineStr">
         <is>
           <t>s01-i3</t>
@@ -957,7 +1006,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="16" customHeight="1" s="7">
+    <row r="18" ht="16" customHeight="1" s="10">
       <c r="A18" s="3" t="inlineStr">
         <is>
           <t>s01-i4</t>
@@ -989,7 +1038,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="16" customHeight="1" s="7">
+    <row r="19" ht="16" customHeight="1" s="10">
       <c r="A19" s="3" t="inlineStr">
         <is>
           <t>s01-i5</t>
@@ -1021,7 +1070,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="16" customHeight="1" s="7">
+    <row r="20" ht="16" customHeight="1" s="10">
       <c r="A20" s="3" t="inlineStr">
         <is>
           <t>s02-title</t>
@@ -1053,7 +1102,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="16" customHeight="1" s="7">
+    <row r="21" ht="16" customHeight="1" s="10">
       <c r="A21" s="3" t="inlineStr">
         <is>
           <t>s02-i1</t>
@@ -1085,7 +1134,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="16" customHeight="1" s="7">
+    <row r="22" ht="16" customHeight="1" s="10">
       <c r="A22" s="3" t="inlineStr">
         <is>
           <t>s02-i2</t>
@@ -1117,7 +1166,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="16" customHeight="1" s="7">
+    <row r="23" ht="16" customHeight="1" s="10">
       <c r="A23" s="3" t="inlineStr">
         <is>
           <t>s02-i3</t>
@@ -1149,7 +1198,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="16" customHeight="1" s="7">
+    <row r="24" ht="16" customHeight="1" s="10">
       <c r="A24" s="3" t="inlineStr">
         <is>
           <t>s02-i4</t>
@@ -1181,7 +1230,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="16" customHeight="1" s="7">
+    <row r="25" ht="16" customHeight="1" s="10">
       <c r="A25" s="3" t="inlineStr">
         <is>
           <t>s02-i5</t>
@@ -1213,7 +1262,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="16" customHeight="1" s="7">
+    <row r="26" ht="16" customHeight="1" s="10">
       <c r="A26" s="3" t="inlineStr">
         <is>
           <t>s03-title</t>
@@ -1245,7 +1294,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="16" customHeight="1" s="7">
+    <row r="27" ht="16" customHeight="1" s="10">
       <c r="A27" s="3" t="inlineStr">
         <is>
           <t>s03-i1</t>
@@ -1277,7 +1326,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="16" customHeight="1" s="7">
+    <row r="28" ht="16" customHeight="1" s="10">
       <c r="A28" s="3" t="inlineStr">
         <is>
           <t>s03-i2</t>
@@ -1309,7 +1358,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="16" customHeight="1" s="7">
+    <row r="29" ht="16" customHeight="1" s="10">
       <c r="A29" s="3" t="inlineStr">
         <is>
           <t>s03-i3</t>
@@ -1341,7 +1390,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="16" customHeight="1" s="7">
+    <row r="30" ht="16" customHeight="1" s="10">
       <c r="A30" s="3" t="inlineStr">
         <is>
           <t>s03-i4</t>
@@ -1373,7 +1422,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="16" customHeight="1" s="7">
+    <row r="31" ht="16" customHeight="1" s="10">
       <c r="A31" s="3" t="inlineStr">
         <is>
           <t>s03-i5</t>
@@ -1405,7 +1454,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="16" customHeight="1" s="7">
+    <row r="32" ht="16" customHeight="1" s="10">
       <c r="A32" s="3" t="inlineStr">
         <is>
           <t>s03-i6</t>
@@ -1437,7 +1486,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="16" customHeight="1" s="7">
+    <row r="33" ht="16" customHeight="1" s="10">
       <c r="A33" s="3" t="inlineStr">
         <is>
           <t>s03-i7</t>
@@ -1469,7 +1518,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="16" customHeight="1" s="7">
+    <row r="34" ht="16" customHeight="1" s="10">
       <c r="A34" s="3" t="inlineStr">
         <is>
           <t>s04-title</t>
@@ -1501,7 +1550,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="16" customHeight="1" s="7">
+    <row r="35" ht="16" customHeight="1" s="10">
       <c r="A35" s="3" t="inlineStr">
         <is>
           <t>s04-i1</t>
@@ -1533,7 +1582,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="16" customHeight="1" s="7">
+    <row r="36" ht="16" customHeight="1" s="10">
       <c r="A36" s="3" t="inlineStr">
         <is>
           <t>s04-i2</t>
@@ -1565,7 +1614,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="16" customHeight="1" s="7">
+    <row r="37" ht="16" customHeight="1" s="10">
       <c r="A37" s="3" t="inlineStr">
         <is>
           <t>s04-i3</t>
@@ -1597,7 +1646,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="16" customHeight="1" s="7">
+    <row r="38" ht="16" customHeight="1" s="10">
       <c r="A38" s="3" t="inlineStr">
         <is>
           <t>s04-i4</t>
@@ -1629,7 +1678,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="16" customHeight="1" s="7">
+    <row r="39" ht="16" customHeight="1" s="10">
       <c r="A39" s="3" t="inlineStr">
         <is>
           <t>s05-title</t>
@@ -1661,7 +1710,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="16" customHeight="1" s="7">
+    <row r="40" ht="16" customHeight="1" s="10">
       <c r="A40" s="3" t="inlineStr">
         <is>
           <t>s05-i1</t>
@@ -1693,7 +1742,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="16" customHeight="1" s="7">
+    <row r="41" ht="16" customHeight="1" s="10">
       <c r="A41" s="3" t="inlineStr">
         <is>
           <t>s05-i2</t>
@@ -1725,7 +1774,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="16" customHeight="1" s="7">
+    <row r="42" ht="16" customHeight="1" s="10">
       <c r="A42" s="3" t="inlineStr">
         <is>
           <t>s05-i3</t>
@@ -1757,7 +1806,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="16" customHeight="1" s="7">
+    <row r="43" ht="16" customHeight="1" s="10">
       <c r="A43" s="3" t="inlineStr">
         <is>
           <t>s05-i4</t>
@@ -1789,7 +1838,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="16" customHeight="1" s="7">
+    <row r="44" ht="16" customHeight="1" s="10">
       <c r="A44" s="3" t="inlineStr">
         <is>
           <t>s06-title</t>
@@ -1821,7 +1870,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="16" customHeight="1" s="7">
+    <row r="45" ht="16" customHeight="1" s="10">
       <c r="A45" s="3" t="inlineStr">
         <is>
           <t>s06-i1</t>
@@ -1853,7 +1902,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="16" customHeight="1" s="7">
+    <row r="46" ht="16" customHeight="1" s="10">
       <c r="A46" s="3" t="inlineStr">
         <is>
           <t>s06-i2</t>
@@ -1885,7 +1934,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="16" customHeight="1" s="7">
+    <row r="47" ht="16" customHeight="1" s="10">
       <c r="A47" s="3" t="inlineStr">
         <is>
           <t>s06-i3</t>
@@ -1917,7 +1966,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="16" customHeight="1" s="7">
+    <row r="48" ht="16" customHeight="1" s="10">
       <c r="A48" s="3" t="inlineStr">
         <is>
           <t>s06-i4</t>
@@ -1949,7 +1998,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="16" customHeight="1" s="7">
+    <row r="49" ht="16" customHeight="1" s="10">
       <c r="A49" s="3" t="inlineStr">
         <is>
           <t>s07-title</t>
@@ -1981,7 +2030,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="16" customHeight="1" s="7">
+    <row r="50" ht="16" customHeight="1" s="10">
       <c r="A50" s="3" t="inlineStr">
         <is>
           <t>s07-i1</t>
@@ -2013,7 +2062,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="32" customHeight="1" s="7">
+    <row r="51" ht="32" customHeight="1" s="10">
       <c r="A51" s="3" t="inlineStr">
         <is>
           <t>s07-i2</t>
@@ -2045,7 +2094,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="32" customHeight="1" s="7">
+    <row r="52" ht="32" customHeight="1" s="10">
       <c r="A52" s="3" t="inlineStr">
         <is>
           <t>s07-i3</t>
@@ -2077,7 +2126,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="32" customHeight="1" s="7">
+    <row r="53" ht="32" customHeight="1" s="10">
       <c r="A53" s="3" t="inlineStr">
         <is>
           <t>s07-i4</t>
@@ -2109,7 +2158,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="16" customHeight="1" s="7">
+    <row r="54" ht="16" customHeight="1" s="10">
       <c r="A54" s="3" t="inlineStr">
         <is>
           <t>s07-i5</t>
@@ -2141,7 +2190,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="16" customHeight="1" s="7">
+    <row r="55" ht="16" customHeight="1" s="10">
       <c r="A55" s="3" t="inlineStr">
         <is>
           <t>s07-i6</t>
@@ -2173,14 +2222,14 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="20" customHeight="1" s="7">
-      <c r="A56" s="6" t="inlineStr">
+    <row r="56" ht="20" customHeight="1" s="10">
+      <c r="A56" s="9" t="inlineStr">
         <is>
           <t>3 · Il problema</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="16" customHeight="1" s="7">
+    <row r="57" ht="16" customHeight="1" s="10">
       <c r="A57" s="3" t="inlineStr">
         <is>
           <t>stag-problem</t>
@@ -2212,7 +2261,7 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="64" customHeight="1" s="7">
+    <row r="58" ht="64" customHeight="1" s="10">
       <c r="A58" s="3" t="inlineStr">
         <is>
           <t>problem-big</t>
@@ -2244,7 +2293,7 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="16" customHeight="1" s="7">
+    <row r="59" ht="16" customHeight="1" s="10">
       <c r="A59" s="3" t="inlineStr">
         <is>
           <t>prob-tag1</t>
@@ -2276,7 +2325,7 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="64" customHeight="1" s="7">
+    <row r="60" ht="64" customHeight="1" s="10">
       <c r="A60" s="3" t="inlineStr">
         <is>
           <t>prob-txt1</t>
@@ -2308,7 +2357,7 @@
         </is>
       </c>
     </row>
-    <row r="61" ht="16" customHeight="1" s="7">
+    <row r="61" ht="16" customHeight="1" s="10">
       <c r="A61" s="3" t="inlineStr">
         <is>
           <t>prob-tag2</t>
@@ -2340,7 +2389,7 @@
         </is>
       </c>
     </row>
-    <row r="62" ht="64" customHeight="1" s="7">
+    <row r="62" ht="64" customHeight="1" s="10">
       <c r="A62" s="3" t="inlineStr">
         <is>
           <t>prob-txt2</t>
@@ -2372,7 +2421,7 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="16" customHeight="1" s="7">
+    <row r="63" ht="16" customHeight="1" s="10">
       <c r="A63" s="3" t="inlineStr">
         <is>
           <t>prob-tag3</t>
@@ -2404,7 +2453,7 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="64" customHeight="1" s="7">
+    <row r="64" ht="64" customHeight="1" s="10">
       <c r="A64" s="3" t="inlineStr">
         <is>
           <t>prob-txt3</t>
@@ -2436,14 +2485,14 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="20" customHeight="1" s="7">
-      <c r="A65" s="6" t="inlineStr">
+    <row r="65" ht="20" customHeight="1" s="10">
+      <c r="A65" s="9" t="inlineStr">
         <is>
           <t>4 · I numeri</t>
         </is>
       </c>
     </row>
-    <row r="66" ht="16" customHeight="1" s="7">
+    <row r="66" ht="16" customHeight="1" s="10">
       <c r="A66" s="3" t="inlineStr">
         <is>
           <t>stag-numbers</t>
@@ -2454,9 +2503,9 @@
           <t>Our supplier network</t>
         </is>
       </c>
-      <c r="C66" s="4" t="inlineStr">
-        <is>
-          <t>La nostra rete fornitori</t>
+      <c r="C66" s="8" t="inlineStr">
+        <is>
+          <t>I nostri numeri</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
@@ -2475,7 +2524,7 @@
         </is>
       </c>
     </row>
-    <row r="67" ht="32" customHeight="1" s="7">
+    <row r="67" ht="32" customHeight="1" s="10">
       <c r="A67" s="3" t="inlineStr">
         <is>
           <t>num-hl</t>
@@ -2507,7 +2556,7 @@
         </is>
       </c>
     </row>
-    <row r="68" ht="16" customHeight="1" s="7">
+    <row r="68" ht="16" customHeight="1" s="10">
       <c r="A68" s="3" t="inlineStr">
         <is>
           <t>nc-t1</t>
@@ -2539,7 +2588,7 @@
         </is>
       </c>
     </row>
-    <row r="69" ht="16" customHeight="1" s="7">
+    <row r="69" ht="16" customHeight="1" s="10">
       <c r="A69" s="3" t="inlineStr">
         <is>
           <t>nc-d1</t>
@@ -2571,7 +2620,7 @@
         </is>
       </c>
     </row>
-    <row r="70" ht="16" customHeight="1" s="7">
+    <row r="70" ht="16" customHeight="1" s="10">
       <c r="A70" s="3" t="inlineStr">
         <is>
           <t>nc-t2</t>
@@ -2603,7 +2652,7 @@
         </is>
       </c>
     </row>
-    <row r="71" ht="16" customHeight="1" s="7">
+    <row r="71" ht="16" customHeight="1" s="10">
       <c r="A71" s="3" t="inlineStr">
         <is>
           <t>nc-d2</t>
@@ -2635,7 +2684,7 @@
         </is>
       </c>
     </row>
-    <row r="72" ht="16" customHeight="1" s="7">
+    <row r="72" ht="16" customHeight="1" s="10">
       <c r="A72" s="3" t="inlineStr">
         <is>
           <t>nc-t3</t>
@@ -2667,7 +2716,7 @@
         </is>
       </c>
     </row>
-    <row r="73" ht="16" customHeight="1" s="7">
+    <row r="73" ht="16" customHeight="1" s="10">
       <c r="A73" s="3" t="inlineStr">
         <is>
           <t>nc-d3</t>
@@ -2699,7 +2748,7 @@
         </is>
       </c>
     </row>
-    <row r="74" ht="16" customHeight="1" s="7">
+    <row r="74" ht="16" customHeight="1" s="10">
       <c r="A74" s="3" t="inlineStr">
         <is>
           <t>nc-t4</t>
@@ -2731,7 +2780,7 @@
         </is>
       </c>
     </row>
-    <row r="75" ht="16" customHeight="1" s="7">
+    <row r="75" ht="16" customHeight="1" s="10">
       <c r="A75" s="3" t="inlineStr">
         <is>
           <t>nc-d4</t>
@@ -2763,7 +2812,7 @@
         </is>
       </c>
     </row>
-    <row r="76" ht="16" customHeight="1" s="7">
+    <row r="76" ht="16" customHeight="1" s="10">
       <c r="A76" s="3" t="inlineStr">
         <is>
           <t>nc-t5</t>
@@ -2795,7 +2844,7 @@
         </is>
       </c>
     </row>
-    <row r="77" ht="16" customHeight="1" s="7">
+    <row r="77" ht="16" customHeight="1" s="10">
       <c r="A77" s="3" t="inlineStr">
         <is>
           <t>nc-d5</t>
@@ -2827,7 +2876,7 @@
         </is>
       </c>
     </row>
-    <row r="78" ht="16" customHeight="1" s="7">
+    <row r="78" ht="16" customHeight="1" s="10">
       <c r="A78" s="3" t="inlineStr">
         <is>
           <t>nc-t6</t>
@@ -2859,7 +2908,7 @@
         </is>
       </c>
     </row>
-    <row r="79" ht="16" customHeight="1" s="7">
+    <row r="79" ht="16" customHeight="1" s="10">
       <c r="A79" s="3" t="inlineStr">
         <is>
           <t>nc-d6</t>
@@ -2891,14 +2940,14 @@
         </is>
       </c>
     </row>
-    <row r="80" ht="20" customHeight="1" s="7">
-      <c r="A80" s="6" t="inlineStr">
+    <row r="80" ht="20" customHeight="1" s="10">
+      <c r="A80" s="9" t="inlineStr">
         <is>
           <t>5 · Perché funziona</t>
         </is>
       </c>
     </row>
-    <row r="81" ht="16" customHeight="1" s="7">
+    <row r="81" ht="16" customHeight="1" s="10">
       <c r="A81" s="3" t="inlineStr">
         <is>
           <t>stag-why</t>
@@ -2930,7 +2979,7 @@
         </is>
       </c>
     </row>
-    <row r="82" ht="16" customHeight="1" s="7">
+    <row r="82" ht="16" customHeight="1" s="10">
       <c r="A82" s="3" t="inlineStr">
         <is>
           <t>wc-t1</t>
@@ -2962,7 +3011,7 @@
         </is>
       </c>
     </row>
-    <row r="83" ht="64" customHeight="1" s="7">
+    <row r="83" ht="64" customHeight="1" s="10">
       <c r="A83" s="3" t="inlineStr">
         <is>
           <t>wc-b1</t>
@@ -2994,7 +3043,7 @@
         </is>
       </c>
     </row>
-    <row r="84" ht="16" customHeight="1" s="7">
+    <row r="84" ht="16" customHeight="1" s="10">
       <c r="A84" s="3" t="inlineStr">
         <is>
           <t>wc-t2</t>
@@ -3026,7 +3075,7 @@
         </is>
       </c>
     </row>
-    <row r="85" ht="80" customHeight="1" s="7">
+    <row r="85" ht="80" customHeight="1" s="10">
       <c r="A85" s="3" t="inlineStr">
         <is>
           <t>wc-b2</t>
@@ -3058,7 +3107,7 @@
         </is>
       </c>
     </row>
-    <row r="86" ht="16" customHeight="1" s="7">
+    <row r="86" ht="16" customHeight="1" s="10">
       <c r="A86" s="3" t="inlineStr">
         <is>
           <t>wc-t3</t>
@@ -3090,7 +3139,7 @@
         </is>
       </c>
     </row>
-    <row r="87" ht="48" customHeight="1" s="7">
+    <row r="87" ht="48" customHeight="1" s="10">
       <c r="A87" s="3" t="inlineStr">
         <is>
           <t>wc-b3</t>
@@ -3122,7 +3171,7 @@
         </is>
       </c>
     </row>
-    <row r="88" ht="16" customHeight="1" s="7">
+    <row r="88" ht="16" customHeight="1" s="10">
       <c r="A88" s="3" t="inlineStr">
         <is>
           <t>wc-t4</t>
@@ -3154,7 +3203,7 @@
         </is>
       </c>
     </row>
-    <row r="89" ht="96" customHeight="1" s="7">
+    <row r="89" ht="96" customHeight="1" s="10">
       <c r="A89" s="3" t="inlineStr">
         <is>
           <t>wc-b4</t>
@@ -3186,7 +3235,7 @@
         </is>
       </c>
     </row>
-    <row r="90" ht="16" customHeight="1" s="7">
+    <row r="90" ht="16" customHeight="1" s="10">
       <c r="A90" s="3" t="inlineStr">
         <is>
           <t>wc-t5</t>
@@ -3218,7 +3267,7 @@
         </is>
       </c>
     </row>
-    <row r="91" ht="64" customHeight="1" s="7">
+    <row r="91" ht="64" customHeight="1" s="10">
       <c r="A91" s="3" t="inlineStr">
         <is>
           <t>wc-b5</t>
@@ -3250,7 +3299,7 @@
         </is>
       </c>
     </row>
-    <row r="92" ht="16" customHeight="1" s="7">
+    <row r="92" ht="16" customHeight="1" s="10">
       <c r="A92" s="3" t="inlineStr">
         <is>
           <t>wc-t6</t>
@@ -3282,7 +3331,7 @@
         </is>
       </c>
     </row>
-    <row r="93" ht="64" customHeight="1" s="7">
+    <row r="93" ht="64" customHeight="1" s="10">
       <c r="A93" s="3" t="inlineStr">
         <is>
           <t>wc-b6</t>
@@ -3314,14 +3363,14 @@
         </is>
       </c>
     </row>
-    <row r="94" ht="20" customHeight="1" s="7">
-      <c r="A94" s="6" t="inlineStr">
+    <row r="94" ht="20" customHeight="1" s="10">
+      <c r="A94" s="9" t="inlineStr">
         <is>
           <t>6 · Cosa facciamo</t>
         </is>
       </c>
     </row>
-    <row r="95" ht="16" customHeight="1" s="7">
+    <row r="95" ht="16" customHeight="1" s="10">
       <c r="A95" s="3" t="inlineStr">
         <is>
           <t>stag-what</t>
@@ -3353,7 +3402,7 @@
         </is>
       </c>
     </row>
-    <row r="96" ht="32" customHeight="1" s="7">
+    <row r="96" ht="32" customHeight="1" s="10">
       <c r="A96" s="3" t="inlineStr">
         <is>
           <t>sol-hl</t>
@@ -3385,7 +3434,7 @@
         </is>
       </c>
     </row>
-    <row r="97" ht="16" customHeight="1" s="7">
+    <row r="97" ht="16" customHeight="1" s="10">
       <c r="A97" s="3" t="inlineStr">
         <is>
           <t>sol-1</t>
@@ -3417,7 +3466,7 @@
         </is>
       </c>
     </row>
-    <row r="98" ht="16" customHeight="1" s="7">
+    <row r="98" ht="16" customHeight="1" s="10">
       <c r="A98" s="3" t="inlineStr">
         <is>
           <t>sol-2</t>
@@ -3449,7 +3498,7 @@
         </is>
       </c>
     </row>
-    <row r="99" ht="16" customHeight="1" s="7">
+    <row r="99" ht="16" customHeight="1" s="10">
       <c r="A99" s="3" t="inlineStr">
         <is>
           <t>sol-3</t>
@@ -3481,7 +3530,7 @@
         </is>
       </c>
     </row>
-    <row r="100" ht="16" customHeight="1" s="7">
+    <row r="100" ht="16" customHeight="1" s="10">
       <c r="A100" s="3" t="inlineStr">
         <is>
           <t>sol-4</t>
@@ -3513,7 +3562,7 @@
         </is>
       </c>
     </row>
-    <row r="101" ht="32" customHeight="1" s="7">
+    <row r="101" ht="32" customHeight="1" s="10">
       <c r="A101" s="3" t="inlineStr">
         <is>
           <t>sol-5</t>
@@ -3545,7 +3594,7 @@
         </is>
       </c>
     </row>
-    <row r="102" ht="32" customHeight="1" s="7">
+    <row r="102" ht="32" customHeight="1" s="10">
       <c r="A102" s="3" t="inlineStr">
         <is>
           <t>sol-6</t>
@@ -3577,821 +3626,821 @@
         </is>
       </c>
     </row>
-    <row r="103" ht="20" customHeight="1" s="7">
-      <c r="A103" s="6" t="inlineStr">
+    <row r="103" ht="20" customHeight="1" s="10">
+      <c r="A103" s="9" t="inlineStr">
         <is>
           <t>7 · Processo</t>
         </is>
       </c>
     </row>
-    <row r="104" ht="16" customHeight="1" s="7">
+    <row r="104" ht="16" customHeight="1" s="10">
       <c r="A104" s="3" t="inlineStr">
         <is>
           <t>pr-t1</t>
         </is>
       </c>
-      <c r="B104" s="11" t="inlineStr">
+      <c r="B104" s="6" t="inlineStr">
         <is>
           <t>Pre-Construction &amp; Audit</t>
         </is>
       </c>
-      <c r="C104" s="11" t="inlineStr">
+      <c r="C104" s="6" t="inlineStr">
         <is>
           <t>Pre-Construction &amp; Audit</t>
         </is>
       </c>
-      <c r="D104" s="11" t="inlineStr">
+      <c r="D104" s="6" t="inlineStr">
         <is>
           <t>施工前审核</t>
         </is>
       </c>
-      <c r="E104" s="11" t="inlineStr">
+      <c r="E104" s="6" t="inlineStr">
         <is>
           <t>Подготовка и аудит</t>
         </is>
       </c>
-      <c r="F104" s="12" t="inlineStr">
+      <c r="F104" s="7" t="inlineStr">
         <is>
           <t>التحضير والتدقيق</t>
         </is>
       </c>
     </row>
-    <row r="105" ht="16" customHeight="1" s="7">
+    <row r="105" ht="16" customHeight="1" s="10">
       <c r="A105" s="3" t="inlineStr">
         <is>
           <t>pr-i1a</t>
         </is>
       </c>
-      <c r="B105" s="11" t="inlineStr">
+      <c r="B105" s="6" t="inlineStr">
         <is>
           <t>Drawing &amp; spec review</t>
         </is>
       </c>
-      <c r="C105" s="11" t="inlineStr">
+      <c r="C105" s="6" t="inlineStr">
         <is>
           <t>Revisione disegni e capitolati</t>
         </is>
       </c>
-      <c r="D105" s="11" t="inlineStr">
+      <c r="D105" s="6" t="inlineStr">
         <is>
           <t>图纸与规范审查</t>
         </is>
       </c>
-      <c r="E105" s="11" t="inlineStr">
+      <c r="E105" s="6" t="inlineStr">
         <is>
           <t>Проверка чертежей и спецификаций</t>
         </is>
       </c>
-      <c r="F105" s="12" t="inlineStr">
+      <c r="F105" s="7" t="inlineStr">
         <is>
           <t>مراجعة الرسومات والمواصفات</t>
         </is>
       </c>
     </row>
-    <row r="106" ht="16" customHeight="1" s="7">
+    <row r="106" ht="16" customHeight="1" s="10">
       <c r="A106" s="3" t="inlineStr">
         <is>
           <t>pr-i1b</t>
         </is>
       </c>
-      <c r="B106" s="4" t="inlineStr">
+      <c r="B106" s="6" t="inlineStr">
         <is>
           <t>Preliminary Budget</t>
         </is>
       </c>
-      <c r="C106" s="4" t="inlineStr">
+      <c r="C106" s="6" t="inlineStr">
         <is>
           <t>Budget preliminare</t>
         </is>
       </c>
-      <c r="D106" s="4" t="inlineStr">
+      <c r="D106" s="6" t="inlineStr">
         <is>
           <t>初步预算</t>
         </is>
       </c>
-      <c r="E106" s="4" t="inlineStr">
+      <c r="E106" s="6" t="inlineStr">
         <is>
           <t>Предварительный бюджет</t>
         </is>
       </c>
-      <c r="F106" s="5" t="inlineStr">
+      <c r="F106" s="7" t="inlineStr">
         <is>
           <t>الميزانية الأولية</t>
         </is>
       </c>
     </row>
-    <row r="107" ht="16" customHeight="1" s="7">
+    <row r="107" ht="16" customHeight="1" s="10">
       <c r="A107" s="3" t="inlineStr">
         <is>
           <t>pr-i1c</t>
         </is>
       </c>
-      <c r="B107" s="11" t="inlineStr">
+      <c r="B107" s="6" t="inlineStr">
         <is>
           <t>RFI risk log</t>
         </is>
       </c>
-      <c r="C107" s="11" t="inlineStr">
+      <c r="C107" s="6" t="inlineStr">
         <is>
           <t>Registro RFI e rischi</t>
         </is>
       </c>
-      <c r="D107" s="11" t="inlineStr">
+      <c r="D107" s="6" t="inlineStr">
         <is>
           <t>RFI 风险记录</t>
         </is>
       </c>
-      <c r="E107" s="11" t="inlineStr">
+      <c r="E107" s="6" t="inlineStr">
         <is>
           <t>Журнал RFI и рисков</t>
         </is>
       </c>
-      <c r="F107" s="12" t="inlineStr">
+      <c r="F107" s="7" t="inlineStr">
         <is>
           <t>سجل RFI والمخاطر</t>
         </is>
       </c>
     </row>
-    <row r="108" ht="32" customHeight="1" s="7">
+    <row r="108" ht="32" customHeight="1" s="10">
       <c r="A108" s="3" t="inlineStr">
         <is>
           <t>pr-i1d</t>
         </is>
       </c>
-      <c r="B108" s="11" t="inlineStr">
+      <c r="B108" s="6" t="inlineStr">
         <is>
           <t>Value engineering</t>
         </is>
       </c>
-      <c r="C108" s="11" t="inlineStr">
+      <c r="C108" s="6" t="inlineStr">
         <is>
           <t>Value engineering</t>
         </is>
       </c>
-      <c r="D108" s="11" t="inlineStr">
+      <c r="D108" s="6" t="inlineStr">
         <is>
           <t>价值工程</t>
         </is>
       </c>
-      <c r="E108" s="11" t="inlineStr">
+      <c r="E108" s="6" t="inlineStr">
         <is>
           <t>Стоимостной инжиниринг</t>
         </is>
       </c>
-      <c r="F108" s="12" t="inlineStr">
+      <c r="F108" s="7" t="inlineStr">
         <is>
           <t>هندسة القيمة</t>
         </is>
       </c>
     </row>
-    <row r="109" ht="16" customHeight="1" s="7">
+    <row r="109" ht="16" customHeight="1" s="10">
       <c r="A109" s="3" t="inlineStr">
         <is>
           <t>pr-t2</t>
         </is>
       </c>
-      <c r="B109" s="11" t="inlineStr">
+      <c r="B109" s="6" t="inlineStr">
         <is>
           <t>Bid &amp; Buyout</t>
         </is>
       </c>
-      <c r="C109" s="11" t="inlineStr">
+      <c r="C109" s="6" t="inlineStr">
         <is>
           <t>Bid &amp; Buyout</t>
         </is>
       </c>
-      <c r="D109" s="11" t="inlineStr">
+      <c r="D109" s="6" t="inlineStr">
         <is>
           <t>招标与采购</t>
         </is>
       </c>
-      <c r="E109" s="11" t="inlineStr">
+      <c r="E109" s="6" t="inlineStr">
         <is>
           <t>Тендер и закупки</t>
         </is>
       </c>
-      <c r="F109" s="12" t="inlineStr">
+      <c r="F109" s="7" t="inlineStr">
         <is>
           <t>المناقصة والشراء</t>
         </is>
       </c>
     </row>
-    <row r="110" ht="16" customHeight="1" s="7">
+    <row r="110" ht="16" customHeight="1" s="10">
       <c r="A110" s="3" t="inlineStr">
         <is>
           <t>pr-i2a</t>
         </is>
       </c>
-      <c r="B110" s="11" t="inlineStr">
+      <c r="B110" s="6" t="inlineStr">
         <is>
           <t>Bid solicitation</t>
         </is>
       </c>
-      <c r="C110" s="11" t="inlineStr">
-        <is>
-          <t>Bando di gara</t>
-        </is>
-      </c>
-      <c r="D110" s="11" t="inlineStr">
+      <c r="C110" s="8" t="inlineStr">
+        <is>
+          <t>RFQ e Gara</t>
+        </is>
+      </c>
+      <c r="D110" s="6" t="inlineStr">
         <is>
           <t>招标公告</t>
         </is>
       </c>
-      <c r="E110" s="11" t="inlineStr">
+      <c r="E110" s="6" t="inlineStr">
         <is>
           <t>Объявление тендера</t>
         </is>
       </c>
-      <c r="F110" s="12" t="inlineStr">
+      <c r="F110" s="7" t="inlineStr">
         <is>
           <t>طرح المناقصة</t>
         </is>
       </c>
     </row>
-    <row r="111" ht="16" customHeight="1" s="7">
+    <row r="111" ht="16" customHeight="1" s="10">
       <c r="A111" s="3" t="inlineStr">
         <is>
           <t>pr-i2b</t>
         </is>
       </c>
-      <c r="B111" s="11" t="inlineStr">
+      <c r="B111" s="6" t="inlineStr">
         <is>
           <t>Subcontractor prequalification</t>
         </is>
       </c>
-      <c r="C111" s="11" t="inlineStr">
+      <c r="C111" s="6" t="inlineStr">
         <is>
           <t>Prequalifica subappaltatori</t>
         </is>
       </c>
-      <c r="D111" s="11" t="inlineStr">
+      <c r="D111" s="6" t="inlineStr">
         <is>
           <t>分包商预审</t>
         </is>
       </c>
-      <c r="E111" s="11" t="inlineStr">
+      <c r="E111" s="6" t="inlineStr">
         <is>
           <t>Предквалификация субподрядчиков</t>
         </is>
       </c>
-      <c r="F111" s="12" t="inlineStr">
+      <c r="F111" s="7" t="inlineStr">
         <is>
           <t>التأهيل المسبق للمقاولين من الباطن</t>
         </is>
       </c>
     </row>
-    <row r="112" ht="16" customHeight="1" s="7">
+    <row r="112" ht="16" customHeight="1" s="10">
       <c r="A112" s="3" t="inlineStr">
         <is>
           <t>pr-i2c</t>
         </is>
       </c>
-      <c r="B112" s="11" t="inlineStr">
+      <c r="B112" s="6" t="inlineStr">
         <is>
           <t>Bid leveling</t>
         </is>
       </c>
-      <c r="C112" s="11" t="inlineStr">
+      <c r="C112" s="8" t="inlineStr">
+        <is>
+          <t>Procurement ed equalizzazione risultati</t>
+        </is>
+      </c>
+      <c r="D112" s="6" t="inlineStr">
+        <is>
+          <t>报价比选</t>
+        </is>
+      </c>
+      <c r="E112" s="6" t="inlineStr">
         <is>
           <t>Bid leveling</t>
         </is>
       </c>
-      <c r="D112" s="11" t="inlineStr">
-        <is>
-          <t>报价比选</t>
-        </is>
-      </c>
-      <c r="E112" s="11" t="inlineStr">
+      <c r="F112" s="7" t="inlineStr">
         <is>
           <t>Bid leveling</t>
         </is>
       </c>
-      <c r="F112" s="12" t="inlineStr">
-        <is>
-          <t>Bid leveling</t>
-        </is>
-      </c>
-    </row>
-    <row r="113" ht="16" customHeight="1" s="7">
+    </row>
+    <row r="113" ht="16" customHeight="1" s="10">
       <c r="A113" s="3" t="inlineStr">
         <is>
           <t>pr-i2d</t>
         </is>
       </c>
-      <c r="B113" s="11" t="inlineStr">
+      <c r="B113" s="6" t="inlineStr">
         <is>
           <t>Award recommendation</t>
         </is>
       </c>
-      <c r="C113" s="11" t="inlineStr">
-        <is>
-          <t>Proposta di aggiudicazione</t>
-        </is>
-      </c>
-      <c r="D113" s="11" t="inlineStr">
+      <c r="C113" s="8" t="inlineStr">
+        <is>
+          <t>Cost Engineering</t>
+        </is>
+      </c>
+      <c r="D113" s="6" t="inlineStr">
         <is>
           <t>授标建议</t>
         </is>
       </c>
-      <c r="E113" s="11" t="inlineStr">
+      <c r="E113" s="6" t="inlineStr">
         <is>
           <t>Рекомендация по присуждению</t>
         </is>
       </c>
-      <c r="F113" s="12" t="inlineStr">
+      <c r="F113" s="7" t="inlineStr">
         <is>
           <t>توصية الإرساء</t>
         </is>
       </c>
     </row>
-    <row r="114" ht="16" customHeight="1" s="7">
+    <row r="114" ht="16" customHeight="1" s="10">
       <c r="A114" s="3" t="inlineStr">
         <is>
           <t>pr-t3</t>
         </is>
       </c>
-      <c r="B114" s="11" t="inlineStr">
+      <c r="B114" s="6" t="inlineStr">
         <is>
           <t>Contract Award</t>
         </is>
       </c>
-      <c r="C114" s="11" t="inlineStr">
-        <is>
-          <t>Aggiudicazione</t>
-        </is>
-      </c>
-      <c r="D114" s="11" t="inlineStr">
+      <c r="C114" s="8" t="inlineStr">
+        <is>
+          <t>Incarico</t>
+        </is>
+      </c>
+      <c r="D114" s="6" t="inlineStr">
         <is>
           <t>合同授予</t>
         </is>
       </c>
-      <c r="E114" s="11" t="inlineStr">
+      <c r="E114" s="6" t="inlineStr">
         <is>
           <t>Заключение договора</t>
         </is>
       </c>
-      <c r="F114" s="12" t="inlineStr">
+      <c r="F114" s="7" t="inlineStr">
         <is>
           <t>إرساء العقد</t>
         </is>
       </c>
     </row>
-    <row r="115" ht="16" customHeight="1" s="7">
+    <row r="115" ht="16" customHeight="1" s="10">
       <c r="A115" s="3" t="inlineStr">
         <is>
           <t>pr-i3a</t>
         </is>
       </c>
-      <c r="B115" s="11" t="inlineStr">
+      <c r="B115" s="6" t="inlineStr">
         <is>
           <t>Scope of Work review</t>
         </is>
       </c>
-      <c r="C115" s="11" t="inlineStr">
+      <c r="C115" s="6" t="inlineStr">
         <is>
           <t>Revisione Scope of Work</t>
         </is>
       </c>
-      <c r="D115" s="11" t="inlineStr">
+      <c r="D115" s="6" t="inlineStr">
         <is>
           <t>工作范围审查</t>
         </is>
       </c>
-      <c r="E115" s="11" t="inlineStr">
+      <c r="E115" s="6" t="inlineStr">
         <is>
           <t>Проверка объёма работ</t>
         </is>
       </c>
-      <c r="F115" s="12" t="inlineStr">
+      <c r="F115" s="7" t="inlineStr">
         <is>
           <t>مراجعة نطاق العمل</t>
         </is>
       </c>
     </row>
-    <row r="116" ht="16" customHeight="1" s="7">
+    <row r="116" ht="16" customHeight="1" s="10">
       <c r="A116" s="3" t="inlineStr">
         <is>
           <t>pr-i3b</t>
         </is>
       </c>
-      <c r="B116" s="11" t="inlineStr">
+      <c r="B116" s="6" t="inlineStr">
         <is>
           <t>Schedule of Values</t>
         </is>
       </c>
-      <c r="C116" s="11" t="inlineStr">
+      <c r="C116" s="6" t="inlineStr">
         <is>
           <t>Schedule of Values</t>
         </is>
       </c>
-      <c r="D116" s="11" t="inlineStr">
+      <c r="D116" s="6" t="inlineStr">
         <is>
           <t>Schedule of Values</t>
         </is>
       </c>
-      <c r="E116" s="11" t="inlineStr">
+      <c r="E116" s="6" t="inlineStr">
         <is>
           <t>Schedule of Values</t>
         </is>
       </c>
-      <c r="F116" s="12" t="inlineStr">
+      <c r="F116" s="7" t="inlineStr">
         <is>
           <t>Schedule of Values</t>
         </is>
       </c>
     </row>
-    <row r="117" ht="16" customHeight="1" s="7">
+    <row r="117" ht="16" customHeight="1" s="10">
       <c r="A117" s="3" t="inlineStr">
         <is>
           <t>pr-i3c</t>
         </is>
       </c>
-      <c r="B117" s="11" t="inlineStr">
+      <c r="B117" s="6" t="inlineStr">
         <is>
           <t>Liquidated damages</t>
         </is>
       </c>
-      <c r="C117" s="11" t="inlineStr">
-        <is>
-          <t>Penali contrattuali</t>
-        </is>
-      </c>
-      <c r="D117" s="11" t="inlineStr">
+      <c r="C117" s="8" t="inlineStr">
+        <is>
+          <t>Sviluppo con garanzia sulle intenzioni di Design</t>
+        </is>
+      </c>
+      <c r="D117" s="6" t="inlineStr">
         <is>
           <t>违约金</t>
         </is>
       </c>
-      <c r="E117" s="11" t="inlineStr">
+      <c r="E117" s="6" t="inlineStr">
         <is>
           <t>Неустойка</t>
         </is>
       </c>
-      <c r="F117" s="12" t="inlineStr">
+      <c r="F117" s="7" t="inlineStr">
         <is>
           <t>غرامات التأخير</t>
         </is>
       </c>
     </row>
-    <row r="118" ht="16" customHeight="1" s="7">
+    <row r="118" ht="16" customHeight="1" s="10">
       <c r="A118" s="3" t="inlineStr">
         <is>
           <t>pr-i3d</t>
         </is>
       </c>
-      <c r="B118" s="4" t="inlineStr">
+      <c r="B118" s="6" t="inlineStr">
         <is>
           <t>Budget tracking</t>
         </is>
       </c>
-      <c r="C118" s="4" t="inlineStr">
+      <c r="C118" s="6" t="inlineStr">
         <is>
           <t>Budget tracking</t>
         </is>
       </c>
-      <c r="D118" s="4" t="inlineStr">
+      <c r="D118" s="6" t="inlineStr">
         <is>
           <t>预算跟踪</t>
         </is>
       </c>
-      <c r="E118" s="4" t="inlineStr">
+      <c r="E118" s="6" t="inlineStr">
         <is>
           <t>Отслеживание бюджета</t>
         </is>
       </c>
-      <c r="F118" s="5" t="inlineStr">
+      <c r="F118" s="7" t="inlineStr">
         <is>
           <t>تتبع الميزانية</t>
         </is>
       </c>
     </row>
-    <row r="119" ht="16" customHeight="1" s="7">
+    <row r="119" ht="16" customHeight="1" s="10">
       <c r="A119" s="3" t="inlineStr">
         <is>
           <t>pr-t4</t>
         </is>
       </c>
-      <c r="B119" s="4" t="inlineStr">
+      <c r="B119" s="6" t="inlineStr">
         <is>
           <t>Delivery &amp; Site</t>
         </is>
       </c>
-      <c r="C119" s="4" t="inlineStr">
+      <c r="C119" s="6" t="inlineStr">
         <is>
           <t>Delivery &amp; Cantiere</t>
         </is>
       </c>
-      <c r="D119" s="4" t="inlineStr">
+      <c r="D119" s="6" t="inlineStr">
         <is>
           <t>交付与现场</t>
         </is>
       </c>
-      <c r="E119" s="4" t="inlineStr">
+      <c r="E119" s="6" t="inlineStr">
         <is>
           <t>Поставка и объект</t>
         </is>
       </c>
-      <c r="F119" s="5" t="inlineStr">
+      <c r="F119" s="7" t="inlineStr">
         <is>
           <t>التسليم والموقع</t>
         </is>
       </c>
     </row>
-    <row r="120" ht="16" customHeight="1" s="7">
+    <row r="120" ht="16" customHeight="1" s="10">
       <c r="A120" s="3" t="inlineStr">
         <is>
           <t>pr-i4a</t>
         </is>
       </c>
-      <c r="B120" s="4" t="inlineStr">
+      <c r="B120" s="6" t="inlineStr">
         <is>
           <t>Site inspections</t>
         </is>
       </c>
-      <c r="C120" s="4" t="inlineStr">
+      <c r="C120" s="6" t="inlineStr">
         <is>
           <t>Ispezioni in loco</t>
         </is>
       </c>
-      <c r="D120" s="4" t="inlineStr">
+      <c r="D120" s="6" t="inlineStr">
         <is>
           <t>现场检查</t>
         </is>
       </c>
-      <c r="E120" s="4" t="inlineStr">
+      <c r="E120" s="6" t="inlineStr">
         <is>
           <t>Инспекции объекта</t>
         </is>
       </c>
-      <c r="F120" s="5" t="inlineStr">
+      <c r="F120" s="7" t="inlineStr">
         <is>
           <t>عمليات تفتيش الموقع</t>
         </is>
       </c>
     </row>
-    <row r="121" ht="16" customHeight="1" s="7">
+    <row r="121" ht="16" customHeight="1" s="10">
       <c r="A121" s="3" t="inlineStr">
         <is>
           <t>pr-i4b</t>
         </is>
       </c>
-      <c r="B121" s="11" t="inlineStr">
+      <c r="B121" s="6" t="inlineStr">
         <is>
           <t>Progress meetings</t>
         </is>
       </c>
-      <c r="C121" s="11" t="inlineStr">
+      <c r="C121" s="6" t="inlineStr">
         <is>
           <t>Riunioni di avanzamento</t>
         </is>
       </c>
-      <c r="D121" s="11" t="inlineStr">
+      <c r="D121" s="6" t="inlineStr">
         <is>
           <t>进度会议</t>
         </is>
       </c>
-      <c r="E121" s="11" t="inlineStr">
+      <c r="E121" s="6" t="inlineStr">
         <is>
           <t>Совещания по ходу работ</t>
         </is>
       </c>
-      <c r="F121" s="12" t="inlineStr">
+      <c r="F121" s="7" t="inlineStr">
         <is>
           <t>اجتماعات المتابعة</t>
         </is>
       </c>
     </row>
-    <row r="122" ht="16" customHeight="1" s="7">
+    <row r="122" ht="16" customHeight="1" s="10">
       <c r="A122" s="3" t="inlineStr">
         <is>
           <t>pr-i4c</t>
         </is>
       </c>
-      <c r="B122" s="11" t="inlineStr">
+      <c r="B122" s="6" t="inlineStr">
         <is>
           <t>Change order log</t>
         </is>
       </c>
-      <c r="C122" s="11" t="inlineStr">
+      <c r="C122" s="6" t="inlineStr">
         <is>
           <t>Registro varianti</t>
         </is>
       </c>
-      <c r="D122" s="11" t="inlineStr">
+      <c r="D122" s="6" t="inlineStr">
         <is>
           <t>变更单记录</t>
         </is>
       </c>
-      <c r="E122" s="11" t="inlineStr">
+      <c r="E122" s="6" t="inlineStr">
         <is>
           <t>Журнал изменений</t>
         </is>
       </c>
-      <c r="F122" s="12" t="inlineStr">
+      <c r="F122" s="7" t="inlineStr">
         <is>
           <t>سجل أوامر التغيير</t>
         </is>
       </c>
     </row>
-    <row r="123" ht="16" customHeight="1" s="7">
+    <row r="123" ht="16" customHeight="1" s="10">
       <c r="A123" s="3" t="inlineStr">
         <is>
           <t>pr-i4d</t>
         </is>
       </c>
-      <c r="B123" s="4" t="inlineStr">
+      <c r="B123" s="6" t="inlineStr">
         <is>
           <t>Escalation protocol</t>
         </is>
       </c>
-      <c r="C123" s="4" t="inlineStr">
+      <c r="C123" s="6" t="inlineStr">
         <is>
           <t>Protocollo escalation</t>
         </is>
       </c>
-      <c r="D123" s="4" t="inlineStr">
+      <c r="D123" s="6" t="inlineStr">
         <is>
           <t>升级协议</t>
         </is>
       </c>
-      <c r="E123" s="4" t="inlineStr">
+      <c r="E123" s="6" t="inlineStr">
         <is>
           <t>Протокол эскалации</t>
         </is>
       </c>
-      <c r="F123" s="5" t="inlineStr">
+      <c r="F123" s="7" t="inlineStr">
         <is>
           <t>بروتوكول التصعيد</t>
         </is>
       </c>
     </row>
-    <row r="124" ht="16" customHeight="1" s="7">
+    <row r="124" ht="16" customHeight="1" s="10">
       <c r="A124" s="3" t="inlineStr">
         <is>
           <t>pr-t5</t>
         </is>
       </c>
-      <c r="B124" s="11" t="inlineStr">
+      <c r="B124" s="6" t="inlineStr">
         <is>
           <t>Closeout &amp; Turnover</t>
         </is>
       </c>
-      <c r="C124" s="11" t="inlineStr">
+      <c r="C124" s="6" t="inlineStr">
         <is>
           <t>Closeout &amp; Turnover</t>
         </is>
       </c>
-      <c r="D124" s="11" t="inlineStr">
+      <c r="D124" s="6" t="inlineStr">
         <is>
           <t>竣工与移交</t>
         </is>
       </c>
-      <c r="E124" s="11" t="inlineStr">
+      <c r="E124" s="6" t="inlineStr">
         <is>
           <t>Закрытие и передача</t>
         </is>
       </c>
-      <c r="F124" s="12" t="inlineStr">
+      <c r="F124" s="7" t="inlineStr">
         <is>
           <t>الإغلاق والتسليم</t>
         </is>
       </c>
     </row>
-    <row r="125" ht="16" customHeight="1" s="7">
+    <row r="125" ht="16" customHeight="1" s="10">
       <c r="A125" s="3" t="inlineStr">
         <is>
           <t>pr-i5a</t>
         </is>
       </c>
-      <c r="B125" s="11" t="inlineStr">
+      <c r="B125" s="6" t="inlineStr">
         <is>
           <t>Substantial completion</t>
         </is>
       </c>
-      <c r="C125" s="11" t="inlineStr">
+      <c r="C125" s="6" t="inlineStr">
         <is>
           <t>Substantial completion</t>
         </is>
       </c>
-      <c r="D125" s="11" t="inlineStr">
+      <c r="D125" s="6" t="inlineStr">
         <is>
           <t>实质性竣工</t>
         </is>
       </c>
-      <c r="E125" s="11" t="inlineStr">
+      <c r="E125" s="6" t="inlineStr">
         <is>
           <t>Существенное завершение</t>
         </is>
       </c>
-      <c r="F125" s="12" t="inlineStr">
+      <c r="F125" s="7" t="inlineStr">
         <is>
           <t>الإنجاز الجوهري</t>
         </is>
       </c>
     </row>
-    <row r="126" ht="16" customHeight="1" s="7">
+    <row r="126" ht="16" customHeight="1" s="10">
       <c r="A126" s="3" t="inlineStr">
         <is>
           <t>pr-i5b</t>
         </is>
       </c>
-      <c r="B126" s="4" t="inlineStr">
+      <c r="B126" s="6" t="inlineStr">
         <is>
           <t>Punch-list</t>
         </is>
       </c>
-      <c r="C126" s="4" t="inlineStr">
+      <c r="C126" s="6" t="inlineStr">
         <is>
           <t>Punch-list</t>
         </is>
       </c>
-      <c r="D126" s="4" t="inlineStr">
+      <c r="D126" s="6" t="inlineStr">
         <is>
           <t>问题清单</t>
         </is>
       </c>
-      <c r="E126" s="4" t="inlineStr">
+      <c r="E126" s="6" t="inlineStr">
         <is>
           <t>Лист замечаний</t>
         </is>
       </c>
-      <c r="F126" s="5" t="inlineStr">
+      <c r="F126" s="7" t="inlineStr">
         <is>
           <t>قائمة النقاط المعلقة</t>
         </is>
       </c>
     </row>
-    <row r="127" ht="16" customHeight="1" s="7">
+    <row r="127" ht="16" customHeight="1" s="10">
       <c r="A127" s="3" t="inlineStr">
         <is>
           <t>pr-i5c</t>
         </is>
       </c>
-      <c r="B127" s="11" t="inlineStr">
+      <c r="B127" s="6" t="inlineStr">
         <is>
           <t>As-built documentation</t>
         </is>
       </c>
-      <c r="C127" s="11" t="inlineStr">
+      <c r="C127" s="6" t="inlineStr">
         <is>
           <t>Documentazione as-built</t>
         </is>
       </c>
-      <c r="D127" s="11" t="inlineStr">
+      <c r="D127" s="6" t="inlineStr">
         <is>
           <t>竣工图文件</t>
         </is>
       </c>
-      <c r="E127" s="11" t="inlineStr">
+      <c r="E127" s="6" t="inlineStr">
         <is>
           <t>Исполнительная документация</t>
         </is>
       </c>
-      <c r="F127" s="12" t="inlineStr">
+      <c r="F127" s="7" t="inlineStr">
         <is>
           <t>مخططات كما نُفِّذت</t>
         </is>
       </c>
     </row>
-    <row r="128" ht="16" customHeight="1" s="7">
+    <row r="128" ht="16" customHeight="1" s="10">
       <c r="A128" s="3" t="inlineStr">
         <is>
           <t>pr-i5d</t>
         </is>
       </c>
-      <c r="B128" s="11" t="inlineStr">
+      <c r="B128" s="6" t="inlineStr">
         <is>
           <t>Warranty &amp; O&amp;M manuals</t>
         </is>
       </c>
-      <c r="C128" s="11" t="inlineStr">
+      <c r="C128" s="6" t="inlineStr">
         <is>
           <t>Garanzie e manuali O&amp;M</t>
         </is>
       </c>
-      <c r="D128" s="11" t="inlineStr">
+      <c r="D128" s="6" t="inlineStr">
         <is>
           <t>保修与运维手册</t>
         </is>
       </c>
-      <c r="E128" s="11" t="inlineStr">
+      <c r="E128" s="6" t="inlineStr">
         <is>
           <t>Гарантии и руководства по эксплуатации</t>
         </is>
       </c>
-      <c r="F128" s="12" t="inlineStr">
+      <c r="F128" s="7" t="inlineStr">
         <is>
           <t>الضمانات وأدلة التشغيل والصيانة</t>
         </is>
       </c>
     </row>
-    <row r="129" ht="20" customHeight="1" s="7">
-      <c r="A129" s="6" t="inlineStr">
+    <row r="129" ht="20" customHeight="1" s="10">
+      <c r="A129" s="9" t="inlineStr">
         <is>
           <t>8 · Profilo / Founder</t>
         </is>
       </c>
     </row>
-    <row r="130" ht="16" customHeight="1" s="7">
+    <row r="130" ht="16" customHeight="1" s="10">
       <c r="A130" s="3" t="inlineStr">
         <is>
           <t>stag-who</t>
@@ -4423,7 +4472,7 @@
         </is>
       </c>
     </row>
-    <row r="131" ht="409.6" customHeight="1" s="7">
+    <row r="131" ht="409.5" customHeight="1" s="10">
       <c r="A131" s="3" t="inlineStr">
         <is>
           <t>bio</t>
@@ -4455,7 +4504,7 @@
         </is>
       </c>
     </row>
-    <row r="132" ht="16" customHeight="1" s="7">
+    <row r="132" ht="16" customHeight="1" s="10">
       <c r="A132" s="3" t="inlineStr">
         <is>
           <t>stag-clients</t>
@@ -4487,7 +4536,7 @@
         </is>
       </c>
     </row>
-    <row r="133" ht="16" customHeight="1" s="7">
+    <row r="133" ht="16" customHeight="1" s="10">
       <c r="A133" s="3" t="inlineStr">
         <is>
           <t>clients-btn</t>
@@ -4519,14 +4568,14 @@
         </is>
       </c>
     </row>
-    <row r="134" ht="20" customHeight="1" s="7">
-      <c r="A134" s="6" t="inlineStr">
+    <row r="134" ht="20" customHeight="1" s="10">
+      <c r="A134" s="9" t="inlineStr">
         <is>
           <t>9 · Chiusura (CTA)</t>
         </is>
       </c>
     </row>
-    <row r="135" ht="16" customHeight="1" s="7">
+    <row r="135" ht="16" customHeight="1" s="10">
       <c r="A135" s="3" t="inlineStr">
         <is>
           <t>cta-hl-1</t>
@@ -4558,7 +4607,7 @@
         </is>
       </c>
     </row>
-    <row r="136" ht="16" customHeight="1" s="7">
+    <row r="136" ht="16" customHeight="1" s="10">
       <c r="A136" s="3" t="inlineStr">
         <is>
           <t>cta-hl-2</t>
@@ -4590,7 +4639,7 @@
         </is>
       </c>
     </row>
-    <row r="137" ht="16" customHeight="1" s="7">
+    <row r="137" ht="16" customHeight="1" s="10">
       <c r="A137" s="3" t="inlineStr">
         <is>
           <t>cta-sub</t>
@@ -4622,14 +4671,14 @@
         </is>
       </c>
     </row>
-    <row r="138" ht="20" customHeight="1" s="7">
-      <c r="A138" s="6" t="inlineStr">
+    <row r="138" ht="20" customHeight="1" s="10">
+      <c r="A138" s="9" t="inlineStr">
         <is>
           <t>Area riservata (finestra password)</t>
         </is>
       </c>
     </row>
-    <row r="139" ht="16" customHeight="1" s="7">
+    <row r="139" ht="16" customHeight="1" s="10">
       <c r="A139" s="3" t="inlineStr">
         <is>
           <t>pwd-title</t>
@@ -4661,7 +4710,7 @@
         </is>
       </c>
     </row>
-    <row r="140" ht="16" customHeight="1" s="7">
+    <row r="140" ht="16" customHeight="1" s="10">
       <c r="A140" s="3" t="inlineStr">
         <is>
           <t>pwd-placeholder</t>
@@ -4693,7 +4742,7 @@
         </is>
       </c>
     </row>
-    <row r="141" ht="16" customHeight="1" s="7">
+    <row r="141" ht="16" customHeight="1" s="10">
       <c r="A141" s="3" t="inlineStr">
         <is>
           <t>pwd-submit</t>
@@ -4730,8 +4779,8 @@
     <mergeCell ref="A129:F129"/>
     <mergeCell ref="A11:F11"/>
     <mergeCell ref="A138:F138"/>
+    <mergeCell ref="A80:F80"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A80:F80"/>
     <mergeCell ref="A94:F94"/>
     <mergeCell ref="A103:F103"/>
     <mergeCell ref="A134:F134"/>
@@ -4743,4 +4792,152 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" style="10" min="1" max="1"/>
+    <col width="46" customWidth="1" style="10" min="2" max="2"/>
+    <col width="20" customWidth="1" style="10" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="42" customHeight="1" s="10">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Cifre delle statistiche — sezione «La nostra rete fornitori». Uguali in tutte le lingue: modifica SOLO la colonna «Valore». Formati: 50+, 40, €570K, €1.1M, 8–15%, ecc. Non toccare la colonna ID.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>Statistica (dove appare)</t>
+        </is>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>Valore (modifica qui)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>stat-nc-t1</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="inlineStr">
+        <is>
+          <t>Top-tier global clients  /  Clienti globali di primo piano</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>50+</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>stat-nc-t2</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>International awards  /  Premi internazionali</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>40+</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>stat-nc-t3</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>Years of experience  /  Anni di esperienza</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>10+</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>stat-nc-t4</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Documented savings — floor  /  Risparmio documentato — minimo</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>€570K</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>stat-nc-t5</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>Documented savings — ceiling  /  Risparmio documentato — massimo</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>€1.1M</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>stat-nc-t6</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>Average tender savings  /  Risparmio medio in gara</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>8–15%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Review sheet: propagate user IT edits to other languages (green), mark user cells processed (black)
</commit_message>
<xml_diff>
--- a/_review/Potential_Revisione_Traduzioni.xlsx
+++ b/_review/Potential_Revisione_Traduzioni.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,23 +65,46 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <i val="1"/>
-      <color rgb="00666666"/>
+      <color rgb="FF666666"/>
       <sz val="9"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <color rgb="00999999"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color rgb="FF999999"/>
       <sz val="9"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
+      <color theme="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <color rgb="001E7D32"/>
-      <sz val="12"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri (Corpo)"/>
+      <color rgb="001E7D32"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="5">
@@ -103,7 +126,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C71617"/>
+        <fgColor rgb="FFC71617"/>
       </patternFill>
     </fill>
   </fills>
@@ -132,23 +155,24 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="FFDDDDDD"/>
       </left>
       <right style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="FFDDDDDD"/>
       </right>
       <top style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="FFDDDDDD"/>
       </top>
       <bottom style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="FFDDDDDD"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -172,6 +196,11 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -182,13 +211,23 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -558,12 +597,12 @@
   <dimension ref="A1:F141"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" style="10" min="1" max="1"/>
-    <col width="34" customWidth="1" style="10" min="2" max="6"/>
+    <col width="16" customWidth="1" style="13" min="1" max="1"/>
+    <col width="34" customWidth="1" style="13" min="2" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" s="10">
-      <c r="A1" s="11" t="inlineStr">
+    <row r="1" ht="34" customHeight="1" s="13">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>Potential — Revisione traduzioni  ·  Modifica le celle di lingua (non la colonna ID). Le righe rosse sono i titoli di sezione (ordine del sito). Simboli &lt;br&gt;/&lt;em&gt; = a capo/evidenziazioni, lasciarli.</t>
         </is>
@@ -601,14 +640,14 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="20" customHeight="1" s="10">
-      <c r="A3" s="9" t="inlineStr">
+    <row r="3" ht="20" customHeight="1" s="13">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Elementi ricorrenti (scroll, footer)</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="16" customHeight="1" s="10">
+    <row r="4" ht="16" customHeight="1" s="13">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>scroll-down</t>
@@ -640,7 +679,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="16" customHeight="1" s="10">
+    <row r="5" ht="16" customHeight="1" s="13">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>footer-copy</t>
@@ -672,7 +711,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="16" customHeight="1" s="10">
+    <row r="6" ht="16" customHeight="1" s="13">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>footer-privacy</t>
@@ -704,14 +743,14 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="20" customHeight="1" s="10">
-      <c r="A7" s="9" t="inlineStr">
+    <row r="7" ht="20" customHeight="1" s="13">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>1 · Frase d'apertura</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="16" customHeight="1" s="10">
+    <row r="8" ht="16" customHeight="1" s="13">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>intro-hl-1</t>
@@ -743,7 +782,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="16" customHeight="1" s="10">
+    <row r="9" ht="16" customHeight="1" s="13">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>intro-hl-2</t>
@@ -775,7 +814,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="16" customHeight="1" s="10">
+    <row r="10" ht="16" customHeight="1" s="13">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>intro-hl-3</t>
@@ -807,14 +846,14 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="20" customHeight="1" s="10">
-      <c r="A11" s="9" t="inlineStr">
+    <row r="11" ht="20" customHeight="1" s="13">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>2 · Aree di competenza</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="16" customHeight="1" s="10">
+    <row r="12" ht="16" customHeight="1" s="13">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>stag-coverage</t>
@@ -846,7 +885,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="32" customHeight="1" s="10">
+    <row r="13" ht="32" customHeight="1" s="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>sectors-hl</t>
@@ -878,7 +917,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="16" customHeight="1" s="10">
+    <row r="14" ht="16" customHeight="1" s="13">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>s01-title</t>
@@ -910,7 +949,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="16" customHeight="1" s="10">
+    <row r="15" ht="16" customHeight="1" s="13">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>s01-i1</t>
@@ -942,7 +981,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="16" customHeight="1" s="10">
+    <row r="16" ht="16" customHeight="1" s="13">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>s01-i2</t>
@@ -974,7 +1013,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="16" customHeight="1" s="10">
+    <row r="17" ht="16" customHeight="1" s="13">
       <c r="A17" s="3" t="inlineStr">
         <is>
           <t>s01-i3</t>
@@ -1006,7 +1045,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="16" customHeight="1" s="10">
+    <row r="18" ht="16" customHeight="1" s="13">
       <c r="A18" s="3" t="inlineStr">
         <is>
           <t>s01-i4</t>
@@ -1038,7 +1077,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="16" customHeight="1" s="10">
+    <row r="19" ht="16" customHeight="1" s="13">
       <c r="A19" s="3" t="inlineStr">
         <is>
           <t>s01-i5</t>
@@ -1070,7 +1109,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="16" customHeight="1" s="10">
+    <row r="20" ht="16" customHeight="1" s="13">
       <c r="A20" s="3" t="inlineStr">
         <is>
           <t>s02-title</t>
@@ -1102,7 +1141,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="16" customHeight="1" s="10">
+    <row r="21" ht="16" customHeight="1" s="13">
       <c r="A21" s="3" t="inlineStr">
         <is>
           <t>s02-i1</t>
@@ -1134,7 +1173,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="16" customHeight="1" s="10">
+    <row r="22" ht="16" customHeight="1" s="13">
       <c r="A22" s="3" t="inlineStr">
         <is>
           <t>s02-i2</t>
@@ -1166,7 +1205,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="16" customHeight="1" s="10">
+    <row r="23" ht="16" customHeight="1" s="13">
       <c r="A23" s="3" t="inlineStr">
         <is>
           <t>s02-i3</t>
@@ -1198,7 +1237,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="16" customHeight="1" s="10">
+    <row r="24" ht="16" customHeight="1" s="13">
       <c r="A24" s="3" t="inlineStr">
         <is>
           <t>s02-i4</t>
@@ -1230,7 +1269,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="16" customHeight="1" s="10">
+    <row r="25" ht="16" customHeight="1" s="13">
       <c r="A25" s="3" t="inlineStr">
         <is>
           <t>s02-i5</t>
@@ -1262,7 +1301,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="16" customHeight="1" s="10">
+    <row r="26" ht="16" customHeight="1" s="13">
       <c r="A26" s="3" t="inlineStr">
         <is>
           <t>s03-title</t>
@@ -1294,7 +1333,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="16" customHeight="1" s="10">
+    <row r="27" ht="16" customHeight="1" s="13">
       <c r="A27" s="3" t="inlineStr">
         <is>
           <t>s03-i1</t>
@@ -1326,7 +1365,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="16" customHeight="1" s="10">
+    <row r="28" ht="16" customHeight="1" s="13">
       <c r="A28" s="3" t="inlineStr">
         <is>
           <t>s03-i2</t>
@@ -1358,7 +1397,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="16" customHeight="1" s="10">
+    <row r="29" ht="16" customHeight="1" s="13">
       <c r="A29" s="3" t="inlineStr">
         <is>
           <t>s03-i3</t>
@@ -1390,7 +1429,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="16" customHeight="1" s="10">
+    <row r="30" ht="16" customHeight="1" s="13">
       <c r="A30" s="3" t="inlineStr">
         <is>
           <t>s03-i4</t>
@@ -1422,7 +1461,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="16" customHeight="1" s="10">
+    <row r="31" ht="16" customHeight="1" s="13">
       <c r="A31" s="3" t="inlineStr">
         <is>
           <t>s03-i5</t>
@@ -1454,7 +1493,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="16" customHeight="1" s="10">
+    <row r="32" ht="16" customHeight="1" s="13">
       <c r="A32" s="3" t="inlineStr">
         <is>
           <t>s03-i6</t>
@@ -1486,7 +1525,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="16" customHeight="1" s="10">
+    <row r="33" ht="16" customHeight="1" s="13">
       <c r="A33" s="3" t="inlineStr">
         <is>
           <t>s03-i7</t>
@@ -1518,7 +1557,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="16" customHeight="1" s="10">
+    <row r="34" ht="16" customHeight="1" s="13">
       <c r="A34" s="3" t="inlineStr">
         <is>
           <t>s04-title</t>
@@ -1550,7 +1589,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="16" customHeight="1" s="10">
+    <row r="35" ht="16" customHeight="1" s="13">
       <c r="A35" s="3" t="inlineStr">
         <is>
           <t>s04-i1</t>
@@ -1582,7 +1621,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="16" customHeight="1" s="10">
+    <row r="36" ht="16" customHeight="1" s="13">
       <c r="A36" s="3" t="inlineStr">
         <is>
           <t>s04-i2</t>
@@ -1614,7 +1653,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="16" customHeight="1" s="10">
+    <row r="37" ht="16" customHeight="1" s="13">
       <c r="A37" s="3" t="inlineStr">
         <is>
           <t>s04-i3</t>
@@ -1646,7 +1685,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="16" customHeight="1" s="10">
+    <row r="38" ht="16" customHeight="1" s="13">
       <c r="A38" s="3" t="inlineStr">
         <is>
           <t>s04-i4</t>
@@ -1678,7 +1717,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="16" customHeight="1" s="10">
+    <row r="39" ht="16" customHeight="1" s="13">
       <c r="A39" s="3" t="inlineStr">
         <is>
           <t>s05-title</t>
@@ -1710,7 +1749,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="16" customHeight="1" s="10">
+    <row r="40" ht="16" customHeight="1" s="13">
       <c r="A40" s="3" t="inlineStr">
         <is>
           <t>s05-i1</t>
@@ -1742,7 +1781,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="16" customHeight="1" s="10">
+    <row r="41" ht="16" customHeight="1" s="13">
       <c r="A41" s="3" t="inlineStr">
         <is>
           <t>s05-i2</t>
@@ -1774,7 +1813,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="16" customHeight="1" s="10">
+    <row r="42" ht="16" customHeight="1" s="13">
       <c r="A42" s="3" t="inlineStr">
         <is>
           <t>s05-i3</t>
@@ -1806,7 +1845,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="16" customHeight="1" s="10">
+    <row r="43" ht="16" customHeight="1" s="13">
       <c r="A43" s="3" t="inlineStr">
         <is>
           <t>s05-i4</t>
@@ -1838,7 +1877,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="16" customHeight="1" s="10">
+    <row r="44" ht="16" customHeight="1" s="13">
       <c r="A44" s="3" t="inlineStr">
         <is>
           <t>s06-title</t>
@@ -1870,7 +1909,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="16" customHeight="1" s="10">
+    <row r="45" ht="16" customHeight="1" s="13">
       <c r="A45" s="3" t="inlineStr">
         <is>
           <t>s06-i1</t>
@@ -1902,7 +1941,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="16" customHeight="1" s="10">
+    <row r="46" ht="16" customHeight="1" s="13">
       <c r="A46" s="3" t="inlineStr">
         <is>
           <t>s06-i2</t>
@@ -1934,7 +1973,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="16" customHeight="1" s="10">
+    <row r="47" ht="16" customHeight="1" s="13">
       <c r="A47" s="3" t="inlineStr">
         <is>
           <t>s06-i3</t>
@@ -1966,7 +2005,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="16" customHeight="1" s="10">
+    <row r="48" ht="16" customHeight="1" s="13">
       <c r="A48" s="3" t="inlineStr">
         <is>
           <t>s06-i4</t>
@@ -1998,7 +2037,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="16" customHeight="1" s="10">
+    <row r="49" ht="16" customHeight="1" s="13">
       <c r="A49" s="3" t="inlineStr">
         <is>
           <t>s07-title</t>
@@ -2030,7 +2069,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="16" customHeight="1" s="10">
+    <row r="50" ht="16" customHeight="1" s="13">
       <c r="A50" s="3" t="inlineStr">
         <is>
           <t>s07-i1</t>
@@ -2062,7 +2101,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="32" customHeight="1" s="10">
+    <row r="51" ht="32" customHeight="1" s="13">
       <c r="A51" s="3" t="inlineStr">
         <is>
           <t>s07-i2</t>
@@ -2094,7 +2133,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="32" customHeight="1" s="10">
+    <row r="52" ht="32" customHeight="1" s="13">
       <c r="A52" s="3" t="inlineStr">
         <is>
           <t>s07-i3</t>
@@ -2126,7 +2165,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="32" customHeight="1" s="10">
+    <row r="53" ht="32" customHeight="1" s="13">
       <c r="A53" s="3" t="inlineStr">
         <is>
           <t>s07-i4</t>
@@ -2158,7 +2197,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="16" customHeight="1" s="10">
+    <row r="54" ht="16" customHeight="1" s="13">
       <c r="A54" s="3" t="inlineStr">
         <is>
           <t>s07-i5</t>
@@ -2190,7 +2229,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="16" customHeight="1" s="10">
+    <row r="55" ht="16" customHeight="1" s="13">
       <c r="A55" s="3" t="inlineStr">
         <is>
           <t>s07-i6</t>
@@ -2222,14 +2261,14 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="20" customHeight="1" s="10">
-      <c r="A56" s="9" t="inlineStr">
+    <row r="56" ht="20" customHeight="1" s="13">
+      <c r="A56" s="12" t="inlineStr">
         <is>
           <t>3 · Il problema</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="16" customHeight="1" s="10">
+    <row r="57" ht="16" customHeight="1" s="13">
       <c r="A57" s="3" t="inlineStr">
         <is>
           <t>stag-problem</t>
@@ -2261,7 +2300,7 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="64" customHeight="1" s="10">
+    <row r="58" ht="64" customHeight="1" s="13">
       <c r="A58" s="3" t="inlineStr">
         <is>
           <t>problem-big</t>
@@ -2293,7 +2332,7 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="16" customHeight="1" s="10">
+    <row r="59" ht="16" customHeight="1" s="13">
       <c r="A59" s="3" t="inlineStr">
         <is>
           <t>prob-tag1</t>
@@ -2325,7 +2364,7 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="64" customHeight="1" s="10">
+    <row r="60" ht="64" customHeight="1" s="13">
       <c r="A60" s="3" t="inlineStr">
         <is>
           <t>prob-txt1</t>
@@ -2357,7 +2396,7 @@
         </is>
       </c>
     </row>
-    <row r="61" ht="16" customHeight="1" s="10">
+    <row r="61" ht="16" customHeight="1" s="13">
       <c r="A61" s="3" t="inlineStr">
         <is>
           <t>prob-tag2</t>
@@ -2389,7 +2428,7 @@
         </is>
       </c>
     </row>
-    <row r="62" ht="64" customHeight="1" s="10">
+    <row r="62" ht="64" customHeight="1" s="13">
       <c r="A62" s="3" t="inlineStr">
         <is>
           <t>prob-txt2</t>
@@ -2421,7 +2460,7 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="16" customHeight="1" s="10">
+    <row r="63" ht="16" customHeight="1" s="13">
       <c r="A63" s="3" t="inlineStr">
         <is>
           <t>prob-tag3</t>
@@ -2453,7 +2492,7 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="64" customHeight="1" s="10">
+    <row r="64" ht="64" customHeight="1" s="13">
       <c r="A64" s="3" t="inlineStr">
         <is>
           <t>prob-txt3</t>
@@ -2485,46 +2524,46 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="20" customHeight="1" s="10">
-      <c r="A65" s="9" t="inlineStr">
+    <row r="65" ht="20" customHeight="1" s="13">
+      <c r="A65" s="12" t="inlineStr">
         <is>
           <t>4 · I numeri</t>
         </is>
       </c>
     </row>
-    <row r="66" ht="16" customHeight="1" s="10">
+    <row r="66" ht="16" customHeight="1" s="13">
       <c r="A66" s="3" t="inlineStr">
         <is>
           <t>stag-numbers</t>
         </is>
       </c>
-      <c r="B66" s="4" t="inlineStr">
-        <is>
-          <t>Our supplier network</t>
-        </is>
-      </c>
-      <c r="C66" s="8" t="inlineStr">
+      <c r="B66" s="17" t="inlineStr">
+        <is>
+          <t>Our numbers</t>
+        </is>
+      </c>
+      <c r="C66" s="18" t="inlineStr">
         <is>
           <t>I nostri numeri</t>
         </is>
       </c>
-      <c r="D66" s="4" t="inlineStr">
-        <is>
-          <t>我们的供应商网络</t>
-        </is>
-      </c>
-      <c r="E66" s="4" t="inlineStr">
-        <is>
-          <t>Наша сеть поставщиков</t>
-        </is>
-      </c>
-      <c r="F66" s="5" t="inlineStr">
-        <is>
-          <t>شبكة موردينا</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="32" customHeight="1" s="10">
+      <c r="D66" s="17" t="inlineStr">
+        <is>
+          <t>我们的数据</t>
+        </is>
+      </c>
+      <c r="E66" s="17" t="inlineStr">
+        <is>
+          <t>Наши цифры</t>
+        </is>
+      </c>
+      <c r="F66" s="19" t="inlineStr">
+        <is>
+          <t>أرقامنا</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="32" customHeight="1" s="13">
       <c r="A67" s="3" t="inlineStr">
         <is>
           <t>num-hl</t>
@@ -2556,7 +2595,7 @@
         </is>
       </c>
     </row>
-    <row r="68" ht="16" customHeight="1" s="10">
+    <row r="68" ht="16" customHeight="1" s="13">
       <c r="A68" s="3" t="inlineStr">
         <is>
           <t>nc-t1</t>
@@ -2588,7 +2627,7 @@
         </is>
       </c>
     </row>
-    <row r="69" ht="16" customHeight="1" s="10">
+    <row r="69" ht="16" customHeight="1" s="13">
       <c r="A69" s="3" t="inlineStr">
         <is>
           <t>nc-d1</t>
@@ -2620,7 +2659,7 @@
         </is>
       </c>
     </row>
-    <row r="70" ht="16" customHeight="1" s="10">
+    <row r="70" ht="16" customHeight="1" s="13">
       <c r="A70" s="3" t="inlineStr">
         <is>
           <t>nc-t2</t>
@@ -2652,7 +2691,7 @@
         </is>
       </c>
     </row>
-    <row r="71" ht="16" customHeight="1" s="10">
+    <row r="71" ht="16" customHeight="1" s="13">
       <c r="A71" s="3" t="inlineStr">
         <is>
           <t>nc-d2</t>
@@ -2684,7 +2723,7 @@
         </is>
       </c>
     </row>
-    <row r="72" ht="16" customHeight="1" s="10">
+    <row r="72" ht="16" customHeight="1" s="13">
       <c r="A72" s="3" t="inlineStr">
         <is>
           <t>nc-t3</t>
@@ -2716,7 +2755,7 @@
         </is>
       </c>
     </row>
-    <row r="73" ht="16" customHeight="1" s="10">
+    <row r="73" ht="16" customHeight="1" s="13">
       <c r="A73" s="3" t="inlineStr">
         <is>
           <t>nc-d3</t>
@@ -2748,7 +2787,7 @@
         </is>
       </c>
     </row>
-    <row r="74" ht="16" customHeight="1" s="10">
+    <row r="74" ht="16" customHeight="1" s="13">
       <c r="A74" s="3" t="inlineStr">
         <is>
           <t>nc-t4</t>
@@ -2780,7 +2819,7 @@
         </is>
       </c>
     </row>
-    <row r="75" ht="16" customHeight="1" s="10">
+    <row r="75" ht="16" customHeight="1" s="13">
       <c r="A75" s="3" t="inlineStr">
         <is>
           <t>nc-d4</t>
@@ -2812,7 +2851,7 @@
         </is>
       </c>
     </row>
-    <row r="76" ht="16" customHeight="1" s="10">
+    <row r="76" ht="16" customHeight="1" s="13">
       <c r="A76" s="3" t="inlineStr">
         <is>
           <t>nc-t5</t>
@@ -2844,7 +2883,7 @@
         </is>
       </c>
     </row>
-    <row r="77" ht="16" customHeight="1" s="10">
+    <row r="77" ht="16" customHeight="1" s="13">
       <c r="A77" s="3" t="inlineStr">
         <is>
           <t>nc-d5</t>
@@ -2876,7 +2915,7 @@
         </is>
       </c>
     </row>
-    <row r="78" ht="16" customHeight="1" s="10">
+    <row r="78" ht="16" customHeight="1" s="13">
       <c r="A78" s="3" t="inlineStr">
         <is>
           <t>nc-t6</t>
@@ -2908,7 +2947,7 @@
         </is>
       </c>
     </row>
-    <row r="79" ht="16" customHeight="1" s="10">
+    <row r="79" ht="16" customHeight="1" s="13">
       <c r="A79" s="3" t="inlineStr">
         <is>
           <t>nc-d6</t>
@@ -2940,14 +2979,14 @@
         </is>
       </c>
     </row>
-    <row r="80" ht="20" customHeight="1" s="10">
-      <c r="A80" s="9" t="inlineStr">
+    <row r="80" ht="20" customHeight="1" s="13">
+      <c r="A80" s="12" t="inlineStr">
         <is>
           <t>5 · Perché funziona</t>
         </is>
       </c>
     </row>
-    <row r="81" ht="16" customHeight="1" s="10">
+    <row r="81" ht="16" customHeight="1" s="13">
       <c r="A81" s="3" t="inlineStr">
         <is>
           <t>stag-why</t>
@@ -2979,7 +3018,7 @@
         </is>
       </c>
     </row>
-    <row r="82" ht="16" customHeight="1" s="10">
+    <row r="82" ht="16" customHeight="1" s="13">
       <c r="A82" s="3" t="inlineStr">
         <is>
           <t>wc-t1</t>
@@ -3011,7 +3050,7 @@
         </is>
       </c>
     </row>
-    <row r="83" ht="64" customHeight="1" s="10">
+    <row r="83" ht="64" customHeight="1" s="13">
       <c r="A83" s="3" t="inlineStr">
         <is>
           <t>wc-b1</t>
@@ -3043,7 +3082,7 @@
         </is>
       </c>
     </row>
-    <row r="84" ht="16" customHeight="1" s="10">
+    <row r="84" ht="16" customHeight="1" s="13">
       <c r="A84" s="3" t="inlineStr">
         <is>
           <t>wc-t2</t>
@@ -3075,7 +3114,7 @@
         </is>
       </c>
     </row>
-    <row r="85" ht="80" customHeight="1" s="10">
+    <row r="85" ht="80" customHeight="1" s="13">
       <c r="A85" s="3" t="inlineStr">
         <is>
           <t>wc-b2</t>
@@ -3107,7 +3146,7 @@
         </is>
       </c>
     </row>
-    <row r="86" ht="16" customHeight="1" s="10">
+    <row r="86" ht="16" customHeight="1" s="13">
       <c r="A86" s="3" t="inlineStr">
         <is>
           <t>wc-t3</t>
@@ -3139,7 +3178,7 @@
         </is>
       </c>
     </row>
-    <row r="87" ht="48" customHeight="1" s="10">
+    <row r="87" ht="48" customHeight="1" s="13">
       <c r="A87" s="3" t="inlineStr">
         <is>
           <t>wc-b3</t>
@@ -3171,7 +3210,7 @@
         </is>
       </c>
     </row>
-    <row r="88" ht="16" customHeight="1" s="10">
+    <row r="88" ht="16" customHeight="1" s="13">
       <c r="A88" s="3" t="inlineStr">
         <is>
           <t>wc-t4</t>
@@ -3203,7 +3242,7 @@
         </is>
       </c>
     </row>
-    <row r="89" ht="96" customHeight="1" s="10">
+    <row r="89" ht="96" customHeight="1" s="13">
       <c r="A89" s="3" t="inlineStr">
         <is>
           <t>wc-b4</t>
@@ -3235,7 +3274,7 @@
         </is>
       </c>
     </row>
-    <row r="90" ht="16" customHeight="1" s="10">
+    <row r="90" ht="16" customHeight="1" s="13">
       <c r="A90" s="3" t="inlineStr">
         <is>
           <t>wc-t5</t>
@@ -3267,7 +3306,7 @@
         </is>
       </c>
     </row>
-    <row r="91" ht="64" customHeight="1" s="10">
+    <row r="91" ht="64" customHeight="1" s="13">
       <c r="A91" s="3" t="inlineStr">
         <is>
           <t>wc-b5</t>
@@ -3299,7 +3338,7 @@
         </is>
       </c>
     </row>
-    <row r="92" ht="16" customHeight="1" s="10">
+    <row r="92" ht="16" customHeight="1" s="13">
       <c r="A92" s="3" t="inlineStr">
         <is>
           <t>wc-t6</t>
@@ -3331,7 +3370,7 @@
         </is>
       </c>
     </row>
-    <row r="93" ht="64" customHeight="1" s="10">
+    <row r="93" ht="64" customHeight="1" s="13">
       <c r="A93" s="3" t="inlineStr">
         <is>
           <t>wc-b6</t>
@@ -3363,14 +3402,14 @@
         </is>
       </c>
     </row>
-    <row r="94" ht="20" customHeight="1" s="10">
-      <c r="A94" s="9" t="inlineStr">
+    <row r="94" ht="20" customHeight="1" s="13">
+      <c r="A94" s="12" t="inlineStr">
         <is>
           <t>6 · Cosa facciamo</t>
         </is>
       </c>
     </row>
-    <row r="95" ht="16" customHeight="1" s="10">
+    <row r="95" ht="16" customHeight="1" s="13">
       <c r="A95" s="3" t="inlineStr">
         <is>
           <t>stag-what</t>
@@ -3402,7 +3441,7 @@
         </is>
       </c>
     </row>
-    <row r="96" ht="32" customHeight="1" s="10">
+    <row r="96" ht="32" customHeight="1" s="13">
       <c r="A96" s="3" t="inlineStr">
         <is>
           <t>sol-hl</t>
@@ -3434,7 +3473,7 @@
         </is>
       </c>
     </row>
-    <row r="97" ht="16" customHeight="1" s="10">
+    <row r="97" ht="16" customHeight="1" s="13">
       <c r="A97" s="3" t="inlineStr">
         <is>
           <t>sol-1</t>
@@ -3466,7 +3505,7 @@
         </is>
       </c>
     </row>
-    <row r="98" ht="16" customHeight="1" s="10">
+    <row r="98" ht="16" customHeight="1" s="13">
       <c r="A98" s="3" t="inlineStr">
         <is>
           <t>sol-2</t>
@@ -3498,7 +3537,7 @@
         </is>
       </c>
     </row>
-    <row r="99" ht="16" customHeight="1" s="10">
+    <row r="99" ht="16" customHeight="1" s="13">
       <c r="A99" s="3" t="inlineStr">
         <is>
           <t>sol-3</t>
@@ -3530,7 +3569,7 @@
         </is>
       </c>
     </row>
-    <row r="100" ht="16" customHeight="1" s="10">
+    <row r="100" ht="16" customHeight="1" s="13">
       <c r="A100" s="3" t="inlineStr">
         <is>
           <t>sol-4</t>
@@ -3562,7 +3601,7 @@
         </is>
       </c>
     </row>
-    <row r="101" ht="32" customHeight="1" s="10">
+    <row r="101" ht="32" customHeight="1" s="13">
       <c r="A101" s="3" t="inlineStr">
         <is>
           <t>sol-5</t>
@@ -3594,7 +3633,7 @@
         </is>
       </c>
     </row>
-    <row r="102" ht="32" customHeight="1" s="10">
+    <row r="102" ht="32" customHeight="1" s="13">
       <c r="A102" s="3" t="inlineStr">
         <is>
           <t>sol-6</t>
@@ -3626,14 +3665,14 @@
         </is>
       </c>
     </row>
-    <row r="103" ht="20" customHeight="1" s="10">
-      <c r="A103" s="9" t="inlineStr">
+    <row r="103" ht="20" customHeight="1" s="13">
+      <c r="A103" s="12" t="inlineStr">
         <is>
           <t>7 · Processo</t>
         </is>
       </c>
     </row>
-    <row r="104" ht="16" customHeight="1" s="10">
+    <row r="104" ht="16" customHeight="1" s="13">
       <c r="A104" s="3" t="inlineStr">
         <is>
           <t>pr-t1</t>
@@ -3665,7 +3704,7 @@
         </is>
       </c>
     </row>
-    <row r="105" ht="16" customHeight="1" s="10">
+    <row r="105" ht="16" customHeight="1" s="13">
       <c r="A105" s="3" t="inlineStr">
         <is>
           <t>pr-i1a</t>
@@ -3697,7 +3736,7 @@
         </is>
       </c>
     </row>
-    <row r="106" ht="16" customHeight="1" s="10">
+    <row r="106" ht="16" customHeight="1" s="13">
       <c r="A106" s="3" t="inlineStr">
         <is>
           <t>pr-i1b</t>
@@ -3729,7 +3768,7 @@
         </is>
       </c>
     </row>
-    <row r="107" ht="16" customHeight="1" s="10">
+    <row r="107" ht="16" customHeight="1" s="13">
       <c r="A107" s="3" t="inlineStr">
         <is>
           <t>pr-i1c</t>
@@ -3761,7 +3800,7 @@
         </is>
       </c>
     </row>
-    <row r="108" ht="32" customHeight="1" s="10">
+    <row r="108" ht="32" customHeight="1" s="13">
       <c r="A108" s="3" t="inlineStr">
         <is>
           <t>pr-i1d</t>
@@ -3793,7 +3832,7 @@
         </is>
       </c>
     </row>
-    <row r="109" ht="16" customHeight="1" s="10">
+    <row r="109" ht="16" customHeight="1" s="13">
       <c r="A109" s="3" t="inlineStr">
         <is>
           <t>pr-t2</t>
@@ -3825,39 +3864,39 @@
         </is>
       </c>
     </row>
-    <row r="110" ht="16" customHeight="1" s="10">
+    <row r="110" ht="16" customHeight="1" s="13">
       <c r="A110" s="3" t="inlineStr">
         <is>
           <t>pr-i2a</t>
         </is>
       </c>
-      <c r="B110" s="6" t="inlineStr">
-        <is>
-          <t>Bid solicitation</t>
-        </is>
-      </c>
-      <c r="C110" s="8" t="inlineStr">
+      <c r="B110" s="20" t="inlineStr">
+        <is>
+          <t>RFQ &amp; tender</t>
+        </is>
+      </c>
+      <c r="C110" s="18" t="inlineStr">
         <is>
           <t>RFQ e Gara</t>
         </is>
       </c>
-      <c r="D110" s="6" t="inlineStr">
-        <is>
-          <t>招标公告</t>
-        </is>
-      </c>
-      <c r="E110" s="6" t="inlineStr">
-        <is>
-          <t>Объявление тендера</t>
-        </is>
-      </c>
-      <c r="F110" s="7" t="inlineStr">
-        <is>
-          <t>طرح المناقصة</t>
-        </is>
-      </c>
-    </row>
-    <row r="111" ht="16" customHeight="1" s="10">
+      <c r="D110" s="20" t="inlineStr">
+        <is>
+          <t>询价与招标</t>
+        </is>
+      </c>
+      <c r="E110" s="20" t="inlineStr">
+        <is>
+          <t>Запрос цен и тендер</t>
+        </is>
+      </c>
+      <c r="F110" s="21" t="inlineStr">
+        <is>
+          <t>طلب عروض الأسعار والمناقصة</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="16" customHeight="1" s="13">
       <c r="A111" s="3" t="inlineStr">
         <is>
           <t>pr-i2b</t>
@@ -3889,71 +3928,71 @@
         </is>
       </c>
     </row>
-    <row r="112" ht="16" customHeight="1" s="10">
+    <row r="112" ht="16" customHeight="1" s="13">
       <c r="A112" s="3" t="inlineStr">
         <is>
           <t>pr-i2c</t>
         </is>
       </c>
-      <c r="B112" s="6" t="inlineStr">
-        <is>
-          <t>Bid leveling</t>
-        </is>
-      </c>
-      <c r="C112" s="8" t="inlineStr">
+      <c r="B112" s="20" t="inlineStr">
+        <is>
+          <t>Procurement &amp; bid leveling</t>
+        </is>
+      </c>
+      <c r="C112" s="18" t="inlineStr">
         <is>
           <t>Procurement ed equalizzazione risultati</t>
         </is>
       </c>
-      <c r="D112" s="6" t="inlineStr">
-        <is>
-          <t>报价比选</t>
-        </is>
-      </c>
-      <c r="E112" s="6" t="inlineStr">
-        <is>
-          <t>Bid leveling</t>
-        </is>
-      </c>
-      <c r="F112" s="7" t="inlineStr">
-        <is>
-          <t>Bid leveling</t>
-        </is>
-      </c>
-    </row>
-    <row r="113" ht="16" customHeight="1" s="10">
+      <c r="D112" s="20" t="inlineStr">
+        <is>
+          <t>采购与报价比选</t>
+        </is>
+      </c>
+      <c r="E112" s="20" t="inlineStr">
+        <is>
+          <t>Закупки и выравнивание предложений</t>
+        </is>
+      </c>
+      <c r="F112" s="21" t="inlineStr">
+        <is>
+          <t>المشتريات وتسوية العطاءات</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="16" customHeight="1" s="13">
       <c r="A113" s="3" t="inlineStr">
         <is>
           <t>pr-i2d</t>
         </is>
       </c>
-      <c r="B113" s="6" t="inlineStr">
-        <is>
-          <t>Award recommendation</t>
-        </is>
-      </c>
-      <c r="C113" s="8" t="inlineStr">
+      <c r="B113" s="20" t="inlineStr">
+        <is>
+          <t>Cost engineering</t>
+        </is>
+      </c>
+      <c r="C113" s="18" t="inlineStr">
         <is>
           <t>Cost Engineering</t>
         </is>
       </c>
-      <c r="D113" s="6" t="inlineStr">
-        <is>
-          <t>授标建议</t>
-        </is>
-      </c>
-      <c r="E113" s="6" t="inlineStr">
-        <is>
-          <t>Рекомендация по присуждению</t>
-        </is>
-      </c>
-      <c r="F113" s="7" t="inlineStr">
-        <is>
-          <t>توصية الإرساء</t>
-        </is>
-      </c>
-    </row>
-    <row r="114" ht="16" customHeight="1" s="10">
+      <c r="D113" s="20" t="inlineStr">
+        <is>
+          <t>成本工程</t>
+        </is>
+      </c>
+      <c r="E113" s="20" t="inlineStr">
+        <is>
+          <t>Стоимостной инжиниринг</t>
+        </is>
+      </c>
+      <c r="F113" s="21" t="inlineStr">
+        <is>
+          <t>هندسة التكلفة</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="16" customHeight="1" s="13">
       <c r="A114" s="3" t="inlineStr">
         <is>
           <t>pr-t3</t>
@@ -3964,7 +4003,7 @@
           <t>Contract Award</t>
         </is>
       </c>
-      <c r="C114" s="8" t="inlineStr">
+      <c r="C114" s="18" t="inlineStr">
         <is>
           <t>Incarico</t>
         </is>
@@ -3985,7 +4024,7 @@
         </is>
       </c>
     </row>
-    <row r="115" ht="16" customHeight="1" s="10">
+    <row r="115" ht="16" customHeight="1" s="13">
       <c r="A115" s="3" t="inlineStr">
         <is>
           <t>pr-i3a</t>
@@ -4017,7 +4056,7 @@
         </is>
       </c>
     </row>
-    <row r="116" ht="16" customHeight="1" s="10">
+    <row r="116" ht="16" customHeight="1" s="13">
       <c r="A116" s="3" t="inlineStr">
         <is>
           <t>pr-i3b</t>
@@ -4049,39 +4088,39 @@
         </is>
       </c>
     </row>
-    <row r="117" ht="16" customHeight="1" s="10">
+    <row r="117" ht="16" customHeight="1" s="13">
       <c r="A117" s="3" t="inlineStr">
         <is>
           <t>pr-i3c</t>
         </is>
       </c>
-      <c r="B117" s="6" t="inlineStr">
-        <is>
-          <t>Liquidated damages</t>
-        </is>
-      </c>
-      <c r="C117" s="8" t="inlineStr">
+      <c r="B117" s="20" t="inlineStr">
+        <is>
+          <t>Design-intent assurance</t>
+        </is>
+      </c>
+      <c r="C117" s="18" t="inlineStr">
         <is>
           <t>Sviluppo con garanzia sulle intenzioni di Design</t>
         </is>
       </c>
-      <c r="D117" s="6" t="inlineStr">
-        <is>
-          <t>违约金</t>
-        </is>
-      </c>
-      <c r="E117" s="6" t="inlineStr">
-        <is>
-          <t>Неустойка</t>
-        </is>
-      </c>
-      <c r="F117" s="7" t="inlineStr">
-        <is>
-          <t>غرامات التأخير</t>
-        </is>
-      </c>
-    </row>
-    <row r="118" ht="16" customHeight="1" s="10">
+      <c r="D117" s="20" t="inlineStr">
+        <is>
+          <t>设计意图保障</t>
+        </is>
+      </c>
+      <c r="E117" s="20" t="inlineStr">
+        <is>
+          <t>Сохранение проектного замысла</t>
+        </is>
+      </c>
+      <c r="F117" s="21" t="inlineStr">
+        <is>
+          <t>ضمان مقصد التصميم</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="16" customHeight="1" s="13">
       <c r="A118" s="3" t="inlineStr">
         <is>
           <t>pr-i3d</t>
@@ -4113,7 +4152,7 @@
         </is>
       </c>
     </row>
-    <row r="119" ht="16" customHeight="1" s="10">
+    <row r="119" ht="16" customHeight="1" s="13">
       <c r="A119" s="3" t="inlineStr">
         <is>
           <t>pr-t4</t>
@@ -4145,7 +4184,7 @@
         </is>
       </c>
     </row>
-    <row r="120" ht="16" customHeight="1" s="10">
+    <row r="120" ht="16" customHeight="1" s="13">
       <c r="A120" s="3" t="inlineStr">
         <is>
           <t>pr-i4a</t>
@@ -4177,7 +4216,7 @@
         </is>
       </c>
     </row>
-    <row r="121" ht="16" customHeight="1" s="10">
+    <row r="121" ht="16" customHeight="1" s="13">
       <c r="A121" s="3" t="inlineStr">
         <is>
           <t>pr-i4b</t>
@@ -4209,7 +4248,7 @@
         </is>
       </c>
     </row>
-    <row r="122" ht="16" customHeight="1" s="10">
+    <row r="122" ht="16" customHeight="1" s="13">
       <c r="A122" s="3" t="inlineStr">
         <is>
           <t>pr-i4c</t>
@@ -4241,7 +4280,7 @@
         </is>
       </c>
     </row>
-    <row r="123" ht="16" customHeight="1" s="10">
+    <row r="123" ht="16" customHeight="1" s="13">
       <c r="A123" s="3" t="inlineStr">
         <is>
           <t>pr-i4d</t>
@@ -4273,7 +4312,7 @@
         </is>
       </c>
     </row>
-    <row r="124" ht="16" customHeight="1" s="10">
+    <row r="124" ht="16" customHeight="1" s="13">
       <c r="A124" s="3" t="inlineStr">
         <is>
           <t>pr-t5</t>
@@ -4305,7 +4344,7 @@
         </is>
       </c>
     </row>
-    <row r="125" ht="16" customHeight="1" s="10">
+    <row r="125" ht="16" customHeight="1" s="13">
       <c r="A125" s="3" t="inlineStr">
         <is>
           <t>pr-i5a</t>
@@ -4337,7 +4376,7 @@
         </is>
       </c>
     </row>
-    <row r="126" ht="16" customHeight="1" s="10">
+    <row r="126" ht="16" customHeight="1" s="13">
       <c r="A126" s="3" t="inlineStr">
         <is>
           <t>pr-i5b</t>
@@ -4369,7 +4408,7 @@
         </is>
       </c>
     </row>
-    <row r="127" ht="16" customHeight="1" s="10">
+    <row r="127" ht="16" customHeight="1" s="13">
       <c r="A127" s="3" t="inlineStr">
         <is>
           <t>pr-i5c</t>
@@ -4401,7 +4440,7 @@
         </is>
       </c>
     </row>
-    <row r="128" ht="16" customHeight="1" s="10">
+    <row r="128" ht="16" customHeight="1" s="13">
       <c r="A128" s="3" t="inlineStr">
         <is>
           <t>pr-i5d</t>
@@ -4433,14 +4472,14 @@
         </is>
       </c>
     </row>
-    <row r="129" ht="20" customHeight="1" s="10">
-      <c r="A129" s="9" t="inlineStr">
+    <row r="129" ht="20" customHeight="1" s="13">
+      <c r="A129" s="12" t="inlineStr">
         <is>
           <t>8 · Profilo / Founder</t>
         </is>
       </c>
     </row>
-    <row r="130" ht="16" customHeight="1" s="10">
+    <row r="130" ht="16" customHeight="1" s="13">
       <c r="A130" s="3" t="inlineStr">
         <is>
           <t>stag-who</t>
@@ -4472,7 +4511,7 @@
         </is>
       </c>
     </row>
-    <row r="131" ht="409.5" customHeight="1" s="10">
+    <row r="131" ht="409.5" customHeight="1" s="13">
       <c r="A131" s="3" t="inlineStr">
         <is>
           <t>bio</t>
@@ -4504,7 +4543,7 @@
         </is>
       </c>
     </row>
-    <row r="132" ht="16" customHeight="1" s="10">
+    <row r="132" ht="16" customHeight="1" s="13">
       <c r="A132" s="3" t="inlineStr">
         <is>
           <t>stag-clients</t>
@@ -4536,7 +4575,7 @@
         </is>
       </c>
     </row>
-    <row r="133" ht="16" customHeight="1" s="10">
+    <row r="133" ht="16" customHeight="1" s="13">
       <c r="A133" s="3" t="inlineStr">
         <is>
           <t>clients-btn</t>
@@ -4568,14 +4607,14 @@
         </is>
       </c>
     </row>
-    <row r="134" ht="20" customHeight="1" s="10">
-      <c r="A134" s="9" t="inlineStr">
+    <row r="134" ht="20" customHeight="1" s="13">
+      <c r="A134" s="12" t="inlineStr">
         <is>
           <t>9 · Chiusura (CTA)</t>
         </is>
       </c>
     </row>
-    <row r="135" ht="16" customHeight="1" s="10">
+    <row r="135" ht="16" customHeight="1" s="13">
       <c r="A135" s="3" t="inlineStr">
         <is>
           <t>cta-hl-1</t>
@@ -4607,7 +4646,7 @@
         </is>
       </c>
     </row>
-    <row r="136" ht="16" customHeight="1" s="10">
+    <row r="136" ht="16" customHeight="1" s="13">
       <c r="A136" s="3" t="inlineStr">
         <is>
           <t>cta-hl-2</t>
@@ -4639,7 +4678,7 @@
         </is>
       </c>
     </row>
-    <row r="137" ht="16" customHeight="1" s="10">
+    <row r="137" ht="16" customHeight="1" s="13">
       <c r="A137" s="3" t="inlineStr">
         <is>
           <t>cta-sub</t>
@@ -4671,14 +4710,14 @@
         </is>
       </c>
     </row>
-    <row r="138" ht="20" customHeight="1" s="10">
-      <c r="A138" s="9" t="inlineStr">
+    <row r="138" ht="20" customHeight="1" s="13">
+      <c r="A138" s="12" t="inlineStr">
         <is>
           <t>Area riservata (finestra password)</t>
         </is>
       </c>
     </row>
-    <row r="139" ht="16" customHeight="1" s="10">
+    <row r="139" ht="16" customHeight="1" s="13">
       <c r="A139" s="3" t="inlineStr">
         <is>
           <t>pwd-title</t>
@@ -4710,7 +4749,7 @@
         </is>
       </c>
     </row>
-    <row r="140" ht="16" customHeight="1" s="10">
+    <row r="140" ht="16" customHeight="1" s="13">
       <c r="A140" s="3" t="inlineStr">
         <is>
           <t>pwd-placeholder</t>
@@ -4742,7 +4781,7 @@
         </is>
       </c>
     </row>
-    <row r="141" ht="16" customHeight="1" s="10">
+    <row r="141" ht="16" customHeight="1" s="13">
       <c r="A141" s="3" t="inlineStr">
         <is>
           <t>pwd-submit</t>
@@ -4779,8 +4818,8 @@
     <mergeCell ref="A129:F129"/>
     <mergeCell ref="A11:F11"/>
     <mergeCell ref="A138:F138"/>
+    <mergeCell ref="A1:F1"/>
     <mergeCell ref="A80:F80"/>
-    <mergeCell ref="A1:F1"/>
     <mergeCell ref="A94:F94"/>
     <mergeCell ref="A103:F103"/>
     <mergeCell ref="A134:F134"/>
@@ -4801,44 +4840,44 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" style="10" min="1" max="1"/>
-    <col width="46" customWidth="1" style="10" min="2" max="2"/>
-    <col width="20" customWidth="1" style="10" min="3" max="3"/>
+    <col width="16" customWidth="1" style="13" min="1" max="1"/>
+    <col width="46" customWidth="1" style="13" min="2" max="2"/>
+    <col width="20" customWidth="1" style="13" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="42" customHeight="1" s="10">
-      <c r="A1" s="12" t="inlineStr">
+    <row r="1" ht="42" customHeight="1" s="13">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Cifre delle statistiche — sezione «La nostra rete fornitori». Uguali in tutte le lingue: modifica SOLO la colonna «Valore». Formati: 50+, 40, €570K, €1.1M, 8–15%, ecc. Non toccare la colonna ID.</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
         <is>
           <t>Statistica (dove appare)</t>
         </is>
       </c>
-      <c r="C2" s="13" t="inlineStr">
+      <c r="C2" s="9" t="inlineStr">
         <is>
           <t>Valore (modifica qui)</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+    <row r="3" ht="16" customHeight="1" s="13">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>stat-nc-t1</t>
         </is>
       </c>
-      <c r="B3" s="15" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Top-tier global clients  /  Clienti globali di primo piano</t>
         </is>
@@ -4849,13 +4888,13 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="14" t="inlineStr">
+    <row r="4" ht="16" customHeight="1" s="13">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>stat-nc-t2</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>International awards  /  Premi internazionali</t>
         </is>
@@ -4866,13 +4905,13 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="14" t="inlineStr">
+    <row r="5" ht="16" customHeight="1" s="13">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>stat-nc-t3</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>Years of experience  /  Anni di esperienza</t>
         </is>
@@ -4883,13 +4922,13 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="14" t="inlineStr">
+    <row r="6" ht="32" customHeight="1" s="13">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>stat-nc-t4</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Documented savings — floor  /  Risparmio documentato — minimo</t>
         </is>
@@ -4900,13 +4939,13 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="14" t="inlineStr">
+    <row r="7" ht="32" customHeight="1" s="13">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>stat-nc-t5</t>
         </is>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Documented savings — ceiling  /  Risparmio documentato — massimo</t>
         </is>
@@ -4917,13 +4956,13 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="14" t="inlineStr">
+    <row r="8" ht="16" customHeight="1" s="13">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>stat-nc-t6</t>
         </is>
       </c>
-      <c r="B8" s="15" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Average tender savings  /  Risparmio medio in gara</t>
         </is>

</xml_diff>

<commit_message>
Review sheet: pr-t3 engagement wording + fix RU value-engineering term (pr-i1d)
</commit_message>
<xml_diff>
--- a/_review/Potential_Revisione_Traduzioni.xlsx
+++ b/_review/Potential_Revisione_Traduzioni.xlsx
@@ -3821,9 +3821,9 @@
           <t>价值工程</t>
         </is>
       </c>
-      <c r="E108" s="6" t="inlineStr">
-        <is>
-          <t>Стоимостной инжиниринг</t>
+      <c r="E108" s="20" t="inlineStr">
+        <is>
+          <t>Функционально-стоимостной инжиниринг</t>
         </is>
       </c>
       <c r="F108" s="7" t="inlineStr">
@@ -3998,9 +3998,9 @@
           <t>pr-t3</t>
         </is>
       </c>
-      <c r="B114" s="6" t="inlineStr">
-        <is>
-          <t>Contract Award</t>
+      <c r="B114" s="20" t="inlineStr">
+        <is>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C114" s="18" t="inlineStr">
@@ -4008,19 +4008,19 @@
           <t>Incarico</t>
         </is>
       </c>
-      <c r="D114" s="6" t="inlineStr">
-        <is>
-          <t>合同授予</t>
-        </is>
-      </c>
-      <c r="E114" s="6" t="inlineStr">
-        <is>
-          <t>Заключение договора</t>
-        </is>
-      </c>
-      <c r="F114" s="7" t="inlineStr">
-        <is>
-          <t>إرساء العقد</t>
+      <c r="D114" s="20" t="inlineStr">
+        <is>
+          <t>委任</t>
+        </is>
+      </c>
+      <c r="E114" s="20" t="inlineStr">
+        <is>
+          <t>Поручение</t>
+        </is>
+      </c>
+      <c r="F114" s="21" t="inlineStr">
+        <is>
+          <t>التكليف</t>
         </is>
       </c>
     </row>
@@ -4818,8 +4818,8 @@
     <mergeCell ref="A129:F129"/>
     <mergeCell ref="A11:F11"/>
     <mergeCell ref="A138:F138"/>
+    <mergeCell ref="A80:F80"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A80:F80"/>
     <mergeCell ref="A94:F94"/>
     <mergeCell ref="A103:F103"/>
     <mergeCell ref="A134:F134"/>

</xml_diff>